<commit_message>
Add InferenceX ingestion layer
</commit_message>
<xml_diff>
--- a/llm_token_capacity_project/outputs/reports/llm_token_capacity_2026_2030.xlsx
+++ b/llm_token_capacity_project/outputs/reports/llm_token_capacity_2026_2030.xlsx
@@ -24,9 +24,13 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08d_benchmark_reference" sheetId="15" state="visible" r:id="rId15"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08e_energy_sanity_reference" sheetId="16" state="visible" r:id="rId16"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="08f_utilization_sensitivity" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_hallucination_checklist" sheetId="18" state="visible" r:id="rId18"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_exec_summary" sheetId="19" state="visible" r:id="rId19"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_charts" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12_inferencex_source_index" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12a_inferencex_schema" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12b_inferencex_tab_rules" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="12c_inferencex_releases" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="11_hallucination_checklist" sheetId="22" state="visible" r:id="rId22"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="09_exec_summary" sheetId="23" state="visible" r:id="rId23"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="10_charts" sheetId="24" state="visible" r:id="rId24"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'00_formula_assumptions'!$A$1:$E$7</definedName>
@@ -46,9 +50,13 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'08d_benchmark_reference'!$A$1:$S$46</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">'08e_energy_sanity_reference'!$A$1:$N$55</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="16" hidden="1">'08f_utilization_sensitivity'!$A$1:$M$73</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="17" hidden="1">'11_hallucination_checklist'!$A$1:$H$16</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="18" hidden="1">'09_exec_summary'!$A$1:$D$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="19" hidden="1">'10_charts'!$A$1:$J$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="17" hidden="1">'12_inferencex_source_index'!$A$1:$AH$11</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="18" hidden="1">'12a_inferencex_schema'!$A$1:$AH$2</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="19" hidden="1">'12b_inferencex_tab_rules'!$A$1:$D$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="20" hidden="1">'12c_inferencex_releases'!$A$1:$K$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="21" hidden="1">'11_hallucination_checklist'!$A$1:$H$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="22" hidden="1">'09_exec_summary'!$A$1:$D$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="23" hidden="1">'10_charts'!$A$1:$J$6</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -36123,693 +36131,859 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H16"/>
+  <dimension ref="A1:AH11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="29" customWidth="1" min="2" max="2"/>
+    <col width="38" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
     <col width="38" customWidth="1" min="3" max="3"/>
-    <col width="38" customWidth="1" min="4" max="4"/>
-    <col width="38" customWidth="1" min="5" max="5"/>
+    <col width="19" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="38" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+    <col width="13" customWidth="1" min="15" max="15"/>
+    <col width="12" customWidth="1" min="16" max="16"/>
+    <col width="13" customWidth="1" min="17" max="17"/>
+    <col width="14" customWidth="1" min="18" max="18"/>
+    <col width="13" customWidth="1" min="19" max="19"/>
+    <col width="12" customWidth="1" min="20" max="20"/>
+    <col width="12" customWidth="1" min="21" max="21"/>
+    <col width="12" customWidth="1" min="22" max="22"/>
+    <col width="17" customWidth="1" min="23" max="23"/>
+    <col width="18" customWidth="1" min="24" max="24"/>
+    <col width="14" customWidth="1" min="25" max="25"/>
+    <col width="13" customWidth="1" min="26" max="26"/>
+    <col width="13" customWidth="1" min="27" max="27"/>
+    <col width="29" customWidth="1" min="28" max="28"/>
+    <col width="12" customWidth="1" min="29" max="29"/>
+    <col width="16" customWidth="1" min="30" max="30"/>
+    <col width="16" customWidth="1" min="31" max="31"/>
+    <col width="38" customWidth="1" min="32" max="32"/>
+    <col width="17" customWidth="1" min="33" max="33"/>
+    <col width="38" customWidth="1" min="34" max="34"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>check_id</t>
+          <t>source_file</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>area</t>
+          <t>source_kind</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>question_kr</t>
+          <t>benchmark_id</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>pass_criteria_kr</t>
+          <t>dashboard_tab</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>risk_if_fail_kr</t>
+          <t>model</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>owner</t>
+          <t>model_family</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>severity</t>
+          <t>gpu</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>current_status</t>
+          <t>gpu_vendor</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>gpu_count</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>framework</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>runtime</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>precision</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>isl</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>osl</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>concurrency</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>batch_size</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>metric_name</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>metric_value</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>metric_unit</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>tok_s_user</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>tok_s_gpu</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>tok_s_mw</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>input_tok_s_gpu</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>output_tok_s_gpu</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>joules_token</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>p99_ttft_ms</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
+          <t>p99_tpot_ms</t>
+        </is>
+      </c>
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
+          <t>cost_per_million_tokens_usd</t>
+        </is>
+      </c>
+      <c r="AC1" s="1" t="inlineStr">
+        <is>
+          <t>power_w</t>
+        </is>
+      </c>
+      <c r="AD1" s="1" t="inlineStr">
+        <is>
+          <t>benchmark_date</t>
+        </is>
+      </c>
+      <c r="AE1" s="1" t="inlineStr">
+        <is>
+          <t>github_run_url</t>
+        </is>
+      </c>
+      <c r="AF1" s="1" t="inlineStr">
+        <is>
+          <t>source_url</t>
+        </is>
+      </c>
+      <c r="AG1" s="1" t="inlineStr">
+        <is>
+          <t>evidence_class</t>
+        </is>
+      </c>
+      <c r="AH1" s="1" t="inlineStr">
+        <is>
+          <t>caveat</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>HC01</t>
+          <t>data/inferencex/raw/INFERENCEX_BENCHMARK_README_README.md</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Source existence</t>
+          <t>benchmark_repo_readme</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>모든 source URL 또는 report name이 실제로 존재하고 접근 가능한가?</t>
+          <t>INFERENCEX_BENCHMARK_README_README</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>01_sources의 URL을 열었을 때 publisher/title/date가 일치한다.</t>
-        </is>
-      </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>없는 출처 또는 잘못된 출처를 근거로 사용.</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>Research</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
-        <is>
-          <t>Needs manual URL click-through</t>
+          <t>methodology</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr"/>
+      <c r="F2" s="2" t="inlineStr"/>
+      <c r="G2" s="2" t="inlineStr"/>
+      <c r="H2" s="2" t="inlineStr"/>
+      <c r="I2" s="2" t="inlineStr"/>
+      <c r="J2" s="2" t="inlineStr"/>
+      <c r="K2" s="2" t="inlineStr"/>
+      <c r="L2" s="2" t="inlineStr"/>
+      <c r="M2" s="2" t="inlineStr"/>
+      <c r="N2" s="2" t="inlineStr"/>
+      <c r="O2" s="2" t="inlineStr"/>
+      <c r="P2" s="2" t="inlineStr"/>
+      <c r="Q2" s="2" t="inlineStr"/>
+      <c r="R2" s="2" t="inlineStr"/>
+      <c r="S2" s="2" t="inlineStr"/>
+      <c r="T2" s="2" t="inlineStr"/>
+      <c r="U2" s="2" t="inlineStr"/>
+      <c r="V2" s="2" t="inlineStr"/>
+      <c r="W2" s="2" t="inlineStr"/>
+      <c r="X2" s="2" t="inlineStr"/>
+      <c r="Y2" s="2" t="inlineStr"/>
+      <c r="Z2" s="2" t="inlineStr"/>
+      <c r="AA2" s="2" t="inlineStr"/>
+      <c r="AB2" s="2" t="inlineStr"/>
+      <c r="AC2" s="2" t="inlineStr"/>
+      <c r="AD2" s="2" t="inlineStr"/>
+      <c r="AE2" s="2" t="inlineStr"/>
+      <c r="AF2" s="2" t="inlineStr">
+        <is>
+          <t>https://github.com/SemiAnalysisAI/InferenceX/blob/main/README.md</t>
+        </is>
+      </c>
+      <c r="AG2" s="2" t="inlineStr">
+        <is>
+          <t>Proxy/Benchmark</t>
+        </is>
+      </c>
+      <c r="AH2" s="2" t="inlineStr">
+        <is>
+          <t>Auto-indexed file-level row; metric values require DB/CSV normalization before use in forecast.</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>HC02</t>
+          <t>data/inferencex/raw/INFERENCEX_BENCHMARK_AGENTS_AGENTS.md</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Numeric fact quote</t>
+          <t>benchmark_repo_operating_rules</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>Fact anchor의 숫자(예: 4.5GW, 671B/37B, 235B/22B, 100k GPU)가 원문에 직접 존재하는가?</t>
+          <t>INFERENCEX_BENCHMARK_AGENTS_AGENTS</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>02a_fact_anchors의 value가 원문 문장/표와 직접 매칭된다.</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>proxy나 추정을 fact처럼 표시.</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>Research</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>Partially checked; requires final source screenshot/quote pack</t>
+          <t>methodology</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr"/>
+      <c r="F3" s="2" t="inlineStr"/>
+      <c r="G3" s="2" t="inlineStr"/>
+      <c r="H3" s="2" t="inlineStr"/>
+      <c r="I3" s="2" t="inlineStr"/>
+      <c r="J3" s="2" t="inlineStr"/>
+      <c r="K3" s="2" t="inlineStr"/>
+      <c r="L3" s="2" t="inlineStr"/>
+      <c r="M3" s="2" t="inlineStr"/>
+      <c r="N3" s="2" t="inlineStr"/>
+      <c r="O3" s="2" t="inlineStr"/>
+      <c r="P3" s="2" t="inlineStr"/>
+      <c r="Q3" s="2" t="inlineStr"/>
+      <c r="R3" s="2" t="inlineStr"/>
+      <c r="S3" s="2" t="inlineStr"/>
+      <c r="T3" s="2" t="inlineStr"/>
+      <c r="U3" s="2" t="inlineStr"/>
+      <c r="V3" s="2" t="inlineStr"/>
+      <c r="W3" s="2" t="inlineStr"/>
+      <c r="X3" s="2" t="inlineStr"/>
+      <c r="Y3" s="2" t="inlineStr"/>
+      <c r="Z3" s="2" t="inlineStr"/>
+      <c r="AA3" s="2" t="inlineStr"/>
+      <c r="AB3" s="2" t="inlineStr"/>
+      <c r="AC3" s="2" t="inlineStr"/>
+      <c r="AD3" s="2" t="inlineStr"/>
+      <c r="AE3" s="2" t="inlineStr"/>
+      <c r="AF3" s="2" t="inlineStr">
+        <is>
+          <t>https://github.com/SemiAnalysisAI/InferenceX/blob/main/AGENTS.md</t>
+        </is>
+      </c>
+      <c r="AG3" s="2" t="inlineStr">
+        <is>
+          <t>Proxy/Benchmark</t>
+        </is>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>Auto-indexed file-level row; metric values require DB/CSV normalization before use in forecast.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>HC03</t>
+          <t>data/inferencex/raw/INFERENCEX_PERF_CHANGELOG_perf-changelog.yaml</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Fact vs estimate separation</t>
+          <t>benchmark_changelog</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>Active GW, inference share, utilization, tokens/sec/MW가 fact로 오표기되지 않았는가?</t>
+          <t>INFERENCEX_PERF_CHANGELOG_perf-changelog</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>해당 값은 Estimate/Scenario로 표시되고 replacement_path가 있다.</t>
-        </is>
-      </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>임원 보고에서 확정 수치처럼 오해.</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>Model</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H4" s="2" t="inlineStr">
-        <is>
-          <t>Pass in structure</t>
+          <t>historical_trends</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr"/>
+      <c r="F4" s="2" t="inlineStr"/>
+      <c r="G4" s="2" t="inlineStr"/>
+      <c r="H4" s="2" t="inlineStr"/>
+      <c r="I4" s="2" t="inlineStr"/>
+      <c r="J4" s="2" t="inlineStr"/>
+      <c r="K4" s="2" t="inlineStr"/>
+      <c r="L4" s="2" t="inlineStr"/>
+      <c r="M4" s="2" t="inlineStr"/>
+      <c r="N4" s="2" t="inlineStr"/>
+      <c r="O4" s="2" t="inlineStr"/>
+      <c r="P4" s="2" t="inlineStr"/>
+      <c r="Q4" s="2" t="inlineStr"/>
+      <c r="R4" s="2" t="inlineStr"/>
+      <c r="S4" s="2" t="inlineStr"/>
+      <c r="T4" s="2" t="inlineStr"/>
+      <c r="U4" s="2" t="inlineStr"/>
+      <c r="V4" s="2" t="inlineStr"/>
+      <c r="W4" s="2" t="inlineStr"/>
+      <c r="X4" s="2" t="inlineStr"/>
+      <c r="Y4" s="2" t="inlineStr"/>
+      <c r="Z4" s="2" t="inlineStr"/>
+      <c r="AA4" s="2" t="inlineStr"/>
+      <c r="AB4" s="2" t="inlineStr"/>
+      <c r="AC4" s="2" t="inlineStr"/>
+      <c r="AD4" s="2" t="inlineStr"/>
+      <c r="AE4" s="2" t="inlineStr"/>
+      <c r="AF4" s="2" t="inlineStr">
+        <is>
+          <t>https://github.com/SemiAnalysisAI/InferenceX/blob/main/perf-changelog.yaml</t>
+        </is>
+      </c>
+      <c r="AG4" s="2" t="inlineStr">
+        <is>
+          <t>Proxy/Benchmark</t>
+        </is>
+      </c>
+      <c r="AH4" s="2" t="inlineStr">
+        <is>
+          <t>Auto-indexed file-level row; metric values require DB/CSV normalization before use in forecast.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>HC04</t>
+          <t>data/inferencex/raw/INFERENCEX_APP_README_README.md</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Closed model parameters</t>
+          <t>dashboard_app_readme</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>OpenAI, Anthropic, Gemini, Grok 같은 closed model에 단일 precise parameter 숫자를 쓰지 않았는가?</t>
+          <t>INFERENCEX_APP_README_README</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>closed model은 band/proxy로만 표시하고 benchmark는 sanity check로만 사용.</t>
-        </is>
-      </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>비공개 파라미터 hallucination.</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>Model</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H5" s="2" t="inlineStr">
-        <is>
-          <t>Pass</t>
+          <t>data_pipeline</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr"/>
+      <c r="F5" s="2" t="inlineStr"/>
+      <c r="G5" s="2" t="inlineStr"/>
+      <c r="H5" s="2" t="inlineStr"/>
+      <c r="I5" s="2" t="inlineStr"/>
+      <c r="J5" s="2" t="inlineStr"/>
+      <c r="K5" s="2" t="inlineStr"/>
+      <c r="L5" s="2" t="inlineStr"/>
+      <c r="M5" s="2" t="inlineStr"/>
+      <c r="N5" s="2" t="inlineStr"/>
+      <c r="O5" s="2" t="inlineStr"/>
+      <c r="P5" s="2" t="inlineStr"/>
+      <c r="Q5" s="2" t="inlineStr"/>
+      <c r="R5" s="2" t="inlineStr"/>
+      <c r="S5" s="2" t="inlineStr"/>
+      <c r="T5" s="2" t="inlineStr"/>
+      <c r="U5" s="2" t="inlineStr"/>
+      <c r="V5" s="2" t="inlineStr"/>
+      <c r="W5" s="2" t="inlineStr"/>
+      <c r="X5" s="2" t="inlineStr"/>
+      <c r="Y5" s="2" t="inlineStr"/>
+      <c r="Z5" s="2" t="inlineStr"/>
+      <c r="AA5" s="2" t="inlineStr"/>
+      <c r="AB5" s="2" t="inlineStr"/>
+      <c r="AC5" s="2" t="inlineStr"/>
+      <c r="AD5" s="2" t="inlineStr"/>
+      <c r="AE5" s="2" t="inlineStr"/>
+      <c r="AF5" s="2" t="inlineStr">
+        <is>
+          <t>https://github.com/SemiAnalysisAI/InferenceX-app/blob/master/README.md</t>
+        </is>
+      </c>
+      <c r="AG5" s="2" t="inlineStr">
+        <is>
+          <t>Proxy/Benchmark</t>
+        </is>
+      </c>
+      <c r="AH5" s="2" t="inlineStr">
+        <is>
+          <t>Auto-indexed file-level row; metric values require DB/CSV normalization before use in forecast.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>HC05</t>
+          <t>data/inferencex/raw/INFERENCEX_APP_ENV_EXAMPLE_.env.example</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>MoE total/active</t>
+          <t>dashboard_app_config</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>MoE 모델은 total params와 active params를 분리했는가?</t>
+          <t>INFERENCEX_APP_ENV_EXAMPLE_.env</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>DeepSeek, Qwen, Llama 4 계열은 total/active가 별도 column 또는 anchor에 존재.</t>
-        </is>
-      </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>MoE 효율을 과소/과대 계산.</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>Model</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="H6" s="2" t="inlineStr">
-        <is>
-          <t>Pass</t>
+          <t>data_pipeline</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr"/>
+      <c r="F6" s="2" t="inlineStr"/>
+      <c r="G6" s="2" t="inlineStr"/>
+      <c r="H6" s="2" t="inlineStr"/>
+      <c r="I6" s="2" t="inlineStr"/>
+      <c r="J6" s="2" t="inlineStr"/>
+      <c r="K6" s="2" t="inlineStr"/>
+      <c r="L6" s="2" t="inlineStr"/>
+      <c r="M6" s="2" t="inlineStr"/>
+      <c r="N6" s="2" t="inlineStr"/>
+      <c r="O6" s="2" t="inlineStr"/>
+      <c r="P6" s="2" t="inlineStr"/>
+      <c r="Q6" s="2" t="inlineStr"/>
+      <c r="R6" s="2" t="inlineStr"/>
+      <c r="S6" s="2" t="inlineStr"/>
+      <c r="T6" s="2" t="inlineStr"/>
+      <c r="U6" s="2" t="inlineStr"/>
+      <c r="V6" s="2" t="inlineStr"/>
+      <c r="W6" s="2" t="inlineStr"/>
+      <c r="X6" s="2" t="inlineStr"/>
+      <c r="Y6" s="2" t="inlineStr"/>
+      <c r="Z6" s="2" t="inlineStr"/>
+      <c r="AA6" s="2" t="inlineStr"/>
+      <c r="AB6" s="2" t="inlineStr"/>
+      <c r="AC6" s="2" t="inlineStr"/>
+      <c r="AD6" s="2" t="inlineStr"/>
+      <c r="AE6" s="2" t="inlineStr"/>
+      <c r="AF6" s="2" t="inlineStr">
+        <is>
+          <t>https://github.com/SemiAnalysisAI/InferenceX-app/blob/master/.env.example</t>
+        </is>
+      </c>
+      <c r="AG6" s="2" t="inlineStr">
+        <is>
+          <t>Proxy/Benchmark</t>
+        </is>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>Auto-indexed file-level row; metric values require DB/CSV normalization before use in forecast.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>HC06</t>
+          <t>data/inferencex/raw/INFERENCEX_APP_PACKAGE_package.json</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Host vs model owner</t>
+          <t>dashboard_app_scripts</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>AWS/Google/Oracle 같은 host capacity가 model owner와 혼동되지 않았는가?</t>
+          <t>INFERENCEX_APP_PACKAGE_package</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Anthropic/OpenAI capacity는 model output 기준으로 귀속하고 host는 source/context로만 표기.</t>
-        </is>
-      </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>capacity double count 또는 wrong attribution.</t>
-        </is>
-      </c>
-      <c r="F7" s="2" t="inlineStr">
-        <is>
-          <t>Model</t>
-        </is>
-      </c>
-      <c r="G7" s="2" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H7" s="2" t="inlineStr">
-        <is>
-          <t>Pass in attribution rules</t>
+          <t>data_pipeline</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr"/>
+      <c r="F7" s="2" t="inlineStr"/>
+      <c r="G7" s="2" t="inlineStr"/>
+      <c r="H7" s="2" t="inlineStr"/>
+      <c r="I7" s="2" t="inlineStr"/>
+      <c r="J7" s="2" t="inlineStr"/>
+      <c r="K7" s="2" t="inlineStr"/>
+      <c r="L7" s="2" t="inlineStr"/>
+      <c r="M7" s="2" t="inlineStr"/>
+      <c r="N7" s="2" t="inlineStr"/>
+      <c r="O7" s="2" t="inlineStr"/>
+      <c r="P7" s="2" t="inlineStr"/>
+      <c r="Q7" s="2" t="inlineStr"/>
+      <c r="R7" s="2" t="inlineStr"/>
+      <c r="S7" s="2" t="inlineStr"/>
+      <c r="T7" s="2" t="inlineStr"/>
+      <c r="U7" s="2" t="inlineStr"/>
+      <c r="V7" s="2" t="inlineStr"/>
+      <c r="W7" s="2" t="inlineStr"/>
+      <c r="X7" s="2" t="inlineStr"/>
+      <c r="Y7" s="2" t="inlineStr"/>
+      <c r="Z7" s="2" t="inlineStr"/>
+      <c r="AA7" s="2" t="inlineStr"/>
+      <c r="AB7" s="2" t="inlineStr"/>
+      <c r="AC7" s="2" t="inlineStr"/>
+      <c r="AD7" s="2" t="inlineStr"/>
+      <c r="AE7" s="2" t="inlineStr"/>
+      <c r="AF7" s="2" t="inlineStr">
+        <is>
+          <t>https://github.com/SemiAnalysisAI/InferenceX-app/blob/master/package.json</t>
+        </is>
+      </c>
+      <c r="AG7" s="2" t="inlineStr">
+        <is>
+          <t>Proxy/Benchmark</t>
+        </is>
+      </c>
+      <c r="AH7" s="2" t="inlineStr">
+        <is>
+          <t>Auto-indexed file-level row; metric values require DB/CSV normalization before use in forecast.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>HC07</t>
+          <t>data/inferencex/raw/INFERENCEX_APP_DATA_PIPELINE_DOC_data-pipeline.md</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Microsoft/OpenAI overlap</t>
+          <t>dashboard_app_doc</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Microsoft Copilot token과 OpenAI model token을 이중계산하지 않았는가?</t>
+          <t>INFERENCEX_APP_DATA_PIPELINE_DOC_data-pipeline</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>OpenAI model output은 OpenAI row, Microsoft-owned/serving burden은 Microsoft row로 명시.</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>OpenAI/Microsoft capacity 중복 산정.</t>
-        </is>
-      </c>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>Model</t>
-        </is>
-      </c>
-      <c r="G8" s="2" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H8" s="2" t="inlineStr">
-        <is>
-          <t>Needs sales/product routing data for final resolution</t>
+          <t>data_pipeline</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr"/>
+      <c r="F8" s="2" t="inlineStr"/>
+      <c r="G8" s="2" t="inlineStr"/>
+      <c r="H8" s="2" t="inlineStr"/>
+      <c r="I8" s="2" t="inlineStr"/>
+      <c r="J8" s="2" t="inlineStr"/>
+      <c r="K8" s="2" t="inlineStr"/>
+      <c r="L8" s="2" t="inlineStr"/>
+      <c r="M8" s="2" t="inlineStr"/>
+      <c r="N8" s="2" t="inlineStr"/>
+      <c r="O8" s="2" t="inlineStr"/>
+      <c r="P8" s="2" t="inlineStr"/>
+      <c r="Q8" s="2" t="inlineStr"/>
+      <c r="R8" s="2" t="inlineStr"/>
+      <c r="S8" s="2" t="inlineStr"/>
+      <c r="T8" s="2" t="inlineStr"/>
+      <c r="U8" s="2" t="inlineStr"/>
+      <c r="V8" s="2" t="inlineStr"/>
+      <c r="W8" s="2" t="inlineStr"/>
+      <c r="X8" s="2" t="inlineStr"/>
+      <c r="Y8" s="2" t="inlineStr"/>
+      <c r="Z8" s="2" t="inlineStr"/>
+      <c r="AA8" s="2" t="inlineStr"/>
+      <c r="AB8" s="2" t="inlineStr"/>
+      <c r="AC8" s="2" t="inlineStr"/>
+      <c r="AD8" s="2" t="inlineStr"/>
+      <c r="AE8" s="2" t="inlineStr"/>
+      <c r="AF8" s="2" t="inlineStr">
+        <is>
+          <t>https://github.com/SemiAnalysisAI/InferenceX-app/blob/master/docs/data-pipeline.md</t>
+        </is>
+      </c>
+      <c r="AG8" s="2" t="inlineStr">
+        <is>
+          <t>Proxy/Benchmark</t>
+        </is>
+      </c>
+      <c r="AH8" s="2" t="inlineStr">
+        <is>
+          <t>Auto-indexed file-level row; metric values require DB/CSV normalization before use in forecast.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>HC08</t>
+          <t>data/inferencex/raw/INFERENCEX_APP_TRANSFORMS_DOC_data-transforms.md</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Capacity boundary</t>
+          <t>dashboard_app_doc</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>active_power_gw가 contracted_power_gw를 넘지 않는가?</t>
+          <t>INFERENCEX_APP_TRANSFORMS_DOC_data-transforms</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>모든 company-year-scenario에서 active &lt;= contracted.</t>
-        </is>
-      </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>물리적으로 불가능한 deployment.</t>
-        </is>
-      </c>
-      <c r="F9" s="2" t="inlineStr">
-        <is>
-          <t>Model</t>
-        </is>
-      </c>
-      <c r="G9" s="2" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H9" s="2" t="inlineStr">
-        <is>
-          <t>Automated pass</t>
+          <t>data_pipeline</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr"/>
+      <c r="F9" s="2" t="inlineStr"/>
+      <c r="G9" s="2" t="inlineStr"/>
+      <c r="H9" s="2" t="inlineStr"/>
+      <c r="I9" s="2" t="inlineStr"/>
+      <c r="J9" s="2" t="inlineStr"/>
+      <c r="K9" s="2" t="inlineStr"/>
+      <c r="L9" s="2" t="inlineStr"/>
+      <c r="M9" s="2" t="inlineStr"/>
+      <c r="N9" s="2" t="inlineStr"/>
+      <c r="O9" s="2" t="inlineStr"/>
+      <c r="P9" s="2" t="inlineStr"/>
+      <c r="Q9" s="2" t="inlineStr"/>
+      <c r="R9" s="2" t="inlineStr"/>
+      <c r="S9" s="2" t="inlineStr"/>
+      <c r="T9" s="2" t="inlineStr"/>
+      <c r="U9" s="2" t="inlineStr"/>
+      <c r="V9" s="2" t="inlineStr"/>
+      <c r="W9" s="2" t="inlineStr"/>
+      <c r="X9" s="2" t="inlineStr"/>
+      <c r="Y9" s="2" t="inlineStr"/>
+      <c r="Z9" s="2" t="inlineStr"/>
+      <c r="AA9" s="2" t="inlineStr"/>
+      <c r="AB9" s="2" t="inlineStr"/>
+      <c r="AC9" s="2" t="inlineStr"/>
+      <c r="AD9" s="2" t="inlineStr"/>
+      <c r="AE9" s="2" t="inlineStr"/>
+      <c r="AF9" s="2" t="inlineStr">
+        <is>
+          <t>https://github.com/SemiAnalysisAI/InferenceX-app/blob/master/docs/data-transforms.md</t>
+        </is>
+      </c>
+      <c r="AG9" s="2" t="inlineStr">
+        <is>
+          <t>Proxy/Benchmark</t>
+        </is>
+      </c>
+      <c r="AH9" s="2" t="inlineStr">
+        <is>
+          <t>Auto-indexed file-level row; metric values require DB/CSV normalization before use in forecast.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>HC09</t>
+          <t>data/inferencex/raw/INFERENCEX_APP_GPU_SPECS_DOC_gpu-specs.md</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Power split</t>
+          <t>dashboard_app_doc</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>training_power_share + inference_power_share = 100%인가?</t>
+          <t>INFERENCEX_APP_GPU_SPECS_DOC_gpu-specs</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>모든 row에서 합계가 1.000 +/- 0.001.</t>
-        </is>
-      </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>GW가 누락 또는 중복.</t>
-        </is>
-      </c>
-      <c r="F10" s="2" t="inlineStr">
-        <is>
-          <t>Model</t>
-        </is>
-      </c>
-      <c r="G10" s="2" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H10" s="2" t="inlineStr">
-        <is>
-          <t>Automated pass</t>
+          <t>gpu_specs</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr"/>
+      <c r="F10" s="2" t="inlineStr"/>
+      <c r="G10" s="2" t="inlineStr"/>
+      <c r="H10" s="2" t="inlineStr"/>
+      <c r="I10" s="2" t="inlineStr"/>
+      <c r="J10" s="2" t="inlineStr"/>
+      <c r="K10" s="2" t="inlineStr"/>
+      <c r="L10" s="2" t="inlineStr"/>
+      <c r="M10" s="2" t="inlineStr"/>
+      <c r="N10" s="2" t="inlineStr"/>
+      <c r="O10" s="2" t="inlineStr"/>
+      <c r="P10" s="2" t="inlineStr"/>
+      <c r="Q10" s="2" t="inlineStr"/>
+      <c r="R10" s="2" t="inlineStr"/>
+      <c r="S10" s="2" t="inlineStr"/>
+      <c r="T10" s="2" t="inlineStr"/>
+      <c r="U10" s="2" t="inlineStr"/>
+      <c r="V10" s="2" t="inlineStr"/>
+      <c r="W10" s="2" t="inlineStr"/>
+      <c r="X10" s="2" t="inlineStr"/>
+      <c r="Y10" s="2" t="inlineStr"/>
+      <c r="Z10" s="2" t="inlineStr"/>
+      <c r="AA10" s="2" t="inlineStr"/>
+      <c r="AB10" s="2" t="inlineStr"/>
+      <c r="AC10" s="2" t="inlineStr"/>
+      <c r="AD10" s="2" t="inlineStr"/>
+      <c r="AE10" s="2" t="inlineStr"/>
+      <c r="AF10" s="2" t="inlineStr">
+        <is>
+          <t>https://github.com/SemiAnalysisAI/InferenceX-app/blob/master/docs/gpu-specs.md</t>
+        </is>
+      </c>
+      <c r="AG10" s="2" t="inlineStr">
+        <is>
+          <t>Proxy/Benchmark</t>
+        </is>
+      </c>
+      <c r="AH10" s="2" t="inlineStr">
+        <is>
+          <t>Auto-indexed file-level row; metric values require DB/CSV normalization before use in forecast.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>HC10</t>
+          <t>data/inferencex/raw/INFERENCEX_APP_TCO_DOC_tco-calculator.md</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Unit consistency</t>
+          <t>dashboard_app_doc</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>daily token과 annual token 단위가 섞이지 않았는가?</t>
+          <t>INFERENCEX_APP_TCO_DOC_tco-calculator</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>token/day는 86,400초, annual token은 365일 또는 31,536,000초로 환산.</t>
-        </is>
-      </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
-          <t>365배 오류 또는 daily/annual 비교 오류.</t>
-        </is>
-      </c>
-      <c r="F11" s="2" t="inlineStr">
-        <is>
-          <t>Model</t>
-        </is>
-      </c>
-      <c r="G11" s="2" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H11" s="2" t="inlineStr">
-        <is>
-          <t>Automated pass</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="2" t="inlineStr">
-        <is>
-          <t>HC11</t>
-        </is>
-      </c>
-      <c r="B12" s="2" t="inlineStr">
-        <is>
-          <t>Benchmark proxy use</t>
-        </is>
-      </c>
-      <c r="C12" s="2" t="inlineStr">
-        <is>
-          <t>OSS/open benchmark를 closed commercial model 결론으로 직접 사용하지 않았는가?</t>
-        </is>
-      </c>
-      <c r="D12" s="2" t="inlineStr">
-        <is>
-          <t>08d_benchmark_reference는 sanity check이며 main forecast와 분리.</t>
-        </is>
-      </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
-          <t>gpt-oss/Qwen/Llama benchmark를 GPT/Claude/Gemini 실서비스로 오인.</t>
-        </is>
-      </c>
-      <c r="F12" s="2" t="inlineStr">
-        <is>
-          <t>Model</t>
-        </is>
-      </c>
-      <c r="G12" s="2" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H12" s="2" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" s="2" t="inlineStr">
-        <is>
-          <t>HC12</t>
-        </is>
-      </c>
-      <c r="B13" s="2" t="inlineStr">
-        <is>
-          <t>Inference share</t>
-        </is>
-      </c>
-      <c r="C13" s="2" t="inlineStr">
-        <is>
-          <t>2026년 추론 60%+를 fact로 단정하지 않았는가?</t>
-        </is>
-      </c>
-      <c r="D13" s="2" t="inlineStr">
-        <is>
-          <t>Base 2026은 60% 미만이고 Bull에서만 60%+ 허용.</t>
-        </is>
-      </c>
-      <c r="E13" s="2" t="inlineStr">
-        <is>
-          <t>전망을 현재 fact처럼 보고.</t>
-        </is>
-      </c>
-      <c r="F13" s="2" t="inlineStr">
-        <is>
-          <t>Model</t>
-        </is>
-      </c>
-      <c r="G13" s="2" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="H13" s="2" t="inlineStr">
-        <is>
-          <t>Pass</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="inlineStr">
-        <is>
-          <t>HC13</t>
-        </is>
-      </c>
-      <c r="B14" s="2" t="inlineStr">
-        <is>
-          <t>Outlier review</t>
-        </is>
-      </c>
-      <c r="C14" s="2" t="inlineStr">
-        <is>
-          <t>main forecast와 benchmark reference의 차이가 큰 업체를 따로 표시했는가?</t>
-        </is>
-      </c>
-      <c r="D14" s="2" t="inlineStr">
-        <is>
-          <t>benchmark_vs_model_pct가 +/-50%를 넘으면 confidence review 대상.</t>
-        </is>
-      </c>
-      <c r="E14" s="2" t="inlineStr">
-        <is>
-          <t>과감한 가정을 숨긴 채 보고.</t>
-        </is>
-      </c>
-      <c r="F14" s="2" t="inlineStr">
-        <is>
-          <t>Model</t>
-        </is>
-      </c>
-      <c r="G14" s="2" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="H14" s="2" t="inlineStr">
-        <is>
-          <t>Needs reviewer sign-off</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>HC14</t>
-        </is>
-      </c>
-      <c r="B15" s="2" t="inlineStr">
-        <is>
-          <t>China transparency</t>
-        </is>
-      </c>
-      <c r="C15" s="2" t="inlineStr">
-        <is>
-          <t>중국 업체의 낮은 공개성 때문에 수치를 임의로 페널티하거나 과신하지 않았는가?</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="inlineStr">
-        <is>
-          <t>모델 구조 fact는 인정하고 capacity transparency만 confidence에 반영.</t>
-        </is>
-      </c>
-      <c r="E15" s="2" t="inlineStr">
-        <is>
-          <t>bias 또는 confidence mislabeling.</t>
-        </is>
-      </c>
-      <c r="F15" s="2" t="inlineStr">
-        <is>
-          <t>Research</t>
-        </is>
-      </c>
-      <c r="G15" s="2" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="H15" s="2" t="inlineStr">
-        <is>
-          <t>Pass in principle; needs Chinese primary-source review</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>HC15</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>Executive wording</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>슬라이드 문구가 추정치를 확정 사실처럼 표현하지 않는가?</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="inlineStr">
-        <is>
-          <t>forecast, scenario, proxy, sanity check, 추정치 표현을 유지.</t>
-        </is>
-      </c>
-      <c r="E16" s="2" t="inlineStr">
-        <is>
-          <t>의사결정자가 불확실성을 과소평가.</t>
-        </is>
-      </c>
-      <c r="F16" s="2" t="inlineStr">
-        <is>
-          <t>Presentation</t>
-        </is>
-      </c>
-      <c r="G16" s="2" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="H16" s="2" t="inlineStr">
-        <is>
-          <t>Needs final human review</t>
+          <t>tco_calculator</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr"/>
+      <c r="F11" s="2" t="inlineStr"/>
+      <c r="G11" s="2" t="inlineStr"/>
+      <c r="H11" s="2" t="inlineStr"/>
+      <c r="I11" s="2" t="inlineStr"/>
+      <c r="J11" s="2" t="inlineStr"/>
+      <c r="K11" s="2" t="inlineStr"/>
+      <c r="L11" s="2" t="inlineStr"/>
+      <c r="M11" s="2" t="inlineStr"/>
+      <c r="N11" s="2" t="inlineStr"/>
+      <c r="O11" s="2" t="inlineStr"/>
+      <c r="P11" s="2" t="inlineStr"/>
+      <c r="Q11" s="2" t="inlineStr"/>
+      <c r="R11" s="2" t="inlineStr"/>
+      <c r="S11" s="2" t="inlineStr"/>
+      <c r="T11" s="2" t="inlineStr"/>
+      <c r="U11" s="2" t="inlineStr"/>
+      <c r="V11" s="2" t="inlineStr"/>
+      <c r="W11" s="2" t="inlineStr"/>
+      <c r="X11" s="2" t="inlineStr"/>
+      <c r="Y11" s="2" t="inlineStr"/>
+      <c r="Z11" s="2" t="inlineStr"/>
+      <c r="AA11" s="2" t="inlineStr"/>
+      <c r="AB11" s="2" t="inlineStr"/>
+      <c r="AC11" s="2" t="inlineStr"/>
+      <c r="AD11" s="2" t="inlineStr"/>
+      <c r="AE11" s="2" t="inlineStr"/>
+      <c r="AF11" s="2" t="inlineStr">
+        <is>
+          <t>https://github.com/SemiAnalysisAI/InferenceX-app/blob/master/docs/tco-calculator.md</t>
+        </is>
+      </c>
+      <c r="AG11" s="2" t="inlineStr">
+        <is>
+          <t>Proxy/Benchmark</t>
+        </is>
+      </c>
+      <c r="AH11" s="2" t="inlineStr">
+        <is>
+          <t>Auto-indexed file-level row; metric values require DB/CSV normalization before use in forecast.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H16"/>
+  <autoFilter ref="A1:AH11"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -36820,197 +36994,255 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:AH2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="38" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="29" customWidth="1" min="3" max="3"/>
-    <col width="38" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="13" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="12" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+    <col width="13" customWidth="1" min="15" max="15"/>
+    <col width="12" customWidth="1" min="16" max="16"/>
+    <col width="13" customWidth="1" min="17" max="17"/>
+    <col width="14" customWidth="1" min="18" max="18"/>
+    <col width="13" customWidth="1" min="19" max="19"/>
+    <col width="12" customWidth="1" min="20" max="20"/>
+    <col width="12" customWidth="1" min="21" max="21"/>
+    <col width="12" customWidth="1" min="22" max="22"/>
+    <col width="17" customWidth="1" min="23" max="23"/>
+    <col width="18" customWidth="1" min="24" max="24"/>
+    <col width="14" customWidth="1" min="25" max="25"/>
+    <col width="13" customWidth="1" min="26" max="26"/>
+    <col width="13" customWidth="1" min="27" max="27"/>
+    <col width="29" customWidth="1" min="28" max="28"/>
+    <col width="12" customWidth="1" min="29" max="29"/>
+    <col width="16" customWidth="1" min="30" max="30"/>
+    <col width="16" customWidth="1" min="31" max="31"/>
+    <col width="12" customWidth="1" min="32" max="32"/>
+    <col width="16" customWidth="1" min="33" max="33"/>
+    <col width="12" customWidth="1" min="34" max="34"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>metric</t>
+          <t>source_file</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>value</t>
+          <t>source_kind</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>display</t>
+          <t>benchmark_id</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>interpretation_kr</t>
+          <t>dashboard_tab</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>model</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>model_family</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>gpu</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>gpu_vendor</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>gpu_count</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>framework</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>runtime</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>precision</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>isl</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>osl</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>concurrency</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>batch_size</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>metric_name</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>metric_value</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>metric_unit</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>tok_s_user</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>tok_s_gpu</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>tok_s_mw</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>input_tok_s_gpu</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>output_tok_s_gpu</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>joules_token</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>p99_ttft_ms</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
+          <t>p99_tpot_ms</t>
+        </is>
+      </c>
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
+          <t>cost_per_million_tokens_usd</t>
+        </is>
+      </c>
+      <c r="AC1" s="1" t="inlineStr">
+        <is>
+          <t>power_w</t>
+        </is>
+      </c>
+      <c r="AD1" s="1" t="inlineStr">
+        <is>
+          <t>benchmark_date</t>
+        </is>
+      </c>
+      <c r="AE1" s="1" t="inlineStr">
+        <is>
+          <t>github_run_url</t>
+        </is>
+      </c>
+      <c r="AF1" s="1" t="inlineStr">
+        <is>
+          <t>source_url</t>
+        </is>
+      </c>
+      <c r="AG1" s="1" t="inlineStr">
+        <is>
+          <t>evidence_class</t>
+        </is>
+      </c>
+      <c r="AH1" s="1" t="inlineStr">
+        <is>
+          <t>caveat</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>2030 core-company inference tokens/day</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="n">
-        <v>2871987625721952</v>
-      </c>
-      <c r="C2" s="2" t="inlineStr">
-        <is>
-          <t>2.87 quadrillion tokens/day</t>
-        </is>
-      </c>
-      <c r="D2" s="2" t="inlineStr">
-        <is>
-          <t>9개 상용 LLM owner의 base case 총 생성 capacity.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>2030 inference AI IT load</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="n">
-        <v>23.02</v>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>23.02 GW inference load</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>PUE와 AI workload share 차감 후 inference에 배정된 IT load.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>2030 US vs China split</t>
-        </is>
-      </c>
-      <c r="B4" s="2" t="inlineStr"/>
-      <c r="C4" s="2" t="inlineStr">
-        <is>
-          <t>US 81% / China 19%</t>
-        </is>
-      </c>
-      <c r="D4" s="2" t="inlineStr">
-        <is>
-          <t>회사 owner 기준 split이며 AWS/Oracle/CoreWeave 같은 host는 core row가 아님.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>Rank 1: OpenAI 2030 tokens/day</t>
-        </is>
-      </c>
-      <c r="B5" s="2" t="n">
-        <v>586840240711296</v>
-      </c>
-      <c r="C5" s="2" t="inlineStr">
-        <is>
-          <t>0.59Q/day</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="inlineStr">
-        <is>
-          <t>GPT / o-series / ChatGPT serving capacity; confidence=Medium</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>Rank 2: Google 2030 tokens/day</t>
-        </is>
-      </c>
-      <c r="B6" s="2" t="n">
-        <v>535132862530560</v>
-      </c>
-      <c r="C6" s="2" t="inlineStr">
-        <is>
-          <t>0.54Q/day</t>
-        </is>
-      </c>
-      <c r="D6" s="2" t="inlineStr">
-        <is>
-          <t>Gemini / Gemma serving capacity; confidence=Medium-High</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>Rank 3: Meta 2030 tokens/day</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="n">
-        <v>402286619750400</v>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>0.40Q/day</t>
-        </is>
-      </c>
-      <c r="D7" s="2" t="inlineStr">
-        <is>
-          <t>Llama / Meta AI serving capacity; confidence=Medium</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>Rank 4: Microsoft 2030 tokens/day</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="n">
-        <v>372288096107136</v>
-      </c>
-      <c r="C8" s="2" t="inlineStr">
-        <is>
-          <t>0.37Q/day</t>
-        </is>
-      </c>
-      <c r="D8" s="2" t="inlineStr">
-        <is>
-          <t>Phi / MAI / Copilot model mix serving capacity; confidence=Medium</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
-        <is>
-          <t>Rank 5: Anthropic 2030 tokens/day</t>
-        </is>
-      </c>
-      <c r="B9" s="2" t="n">
-        <v>318303245151360</v>
-      </c>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>0.32Q/day</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>Claude Opus / Sonnet / Haiku serving capacity; confidence=Medium</t>
-        </is>
-      </c>
+      <c r="A2" s="2" t="inlineStr"/>
+      <c r="B2" s="2" t="inlineStr"/>
+      <c r="C2" s="2" t="inlineStr"/>
+      <c r="D2" s="2" t="inlineStr"/>
+      <c r="E2" s="2" t="inlineStr"/>
+      <c r="F2" s="2" t="inlineStr"/>
+      <c r="G2" s="2" t="inlineStr"/>
+      <c r="H2" s="2" t="inlineStr"/>
+      <c r="I2" s="2" t="inlineStr"/>
+      <c r="J2" s="2" t="inlineStr"/>
+      <c r="K2" s="2" t="inlineStr"/>
+      <c r="L2" s="2" t="inlineStr"/>
+      <c r="M2" s="2" t="inlineStr"/>
+      <c r="N2" s="2" t="inlineStr"/>
+      <c r="O2" s="2" t="inlineStr"/>
+      <c r="P2" s="2" t="inlineStr"/>
+      <c r="Q2" s="2" t="inlineStr"/>
+      <c r="R2" s="2" t="inlineStr"/>
+      <c r="S2" s="2" t="inlineStr"/>
+      <c r="T2" s="2" t="inlineStr"/>
+      <c r="U2" s="2" t="inlineStr"/>
+      <c r="V2" s="2" t="inlineStr"/>
+      <c r="W2" s="2" t="inlineStr"/>
+      <c r="X2" s="2" t="inlineStr"/>
+      <c r="Y2" s="2" t="inlineStr"/>
+      <c r="Z2" s="2" t="inlineStr"/>
+      <c r="AA2" s="2" t="inlineStr"/>
+      <c r="AB2" s="2" t="inlineStr"/>
+      <c r="AC2" s="2" t="inlineStr"/>
+      <c r="AD2" s="2" t="inlineStr"/>
+      <c r="AE2" s="2" t="inlineStr"/>
+      <c r="AF2" s="2" t="inlineStr"/>
+      <c r="AG2" s="2" t="inlineStr"/>
+      <c r="AH2" s="2" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:D9"/>
+  <autoFilter ref="A1:AH2"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -38394,6 +38626,1598 @@
 </file>
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="23" customWidth="1" min="1" max="1"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="38" customWidth="1" min="3" max="3"/>
+    <col width="38" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>dashboard_tab</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>use_in_model</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>required_keys</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>forecast_use</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>inference_performance</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>A08 tokens/sec/MW, A09 latency/utilization sensitivity</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>model, gpu, framework/runtime, precision, ISL, OSL, concurrency, throughput, latency</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>benchmark/proxy only</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>accuracy_evals</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>model quality guardrail when comparing precision/quantization choices</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>model, precision, benchmark, score, date</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>quality sanity check; not token capacity</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>historical_trends</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>software improvement CAGR, SGLang/vLLM/TRT-LLM version step changes</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>config key, software version, benchmark date, PR/run URL</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>scenario support for Bull/Base/Bear tokens/MW improvement</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>tco_calculator</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>cost/token and memory marketing implications</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>GPU, system cost, power, throughput, utilization, amortization</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>commercial sensitivity layer, not production volume</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>gpu_specs</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>GPU generation, memory capacity/bandwidth, TDP cross-check</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>GPU, vendor, memory, bandwidth, power/TDP</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>hardware sanity check for GPU/ASIC mix</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:D6"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="31" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
+    <col width="32" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="38" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="38" customWidth="1" min="9" max="9"/>
+    <col width="38" customWidth="1" min="10" max="10"/>
+    <col width="23" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>repo</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>tag_name</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>published_at</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>asset_name</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>asset_size_bytes</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>asset_digest</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>download_count</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>browser_download_url</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>html_url</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>body</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>SemiAnalysisAI/InferenceX-app</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>db-dump/2026-05-11</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>DB Dump 2026-05-11</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-11T01:11:04Z</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>inferencex-dump-2026-05-11.zip</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>2072340792</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>sha256:3f59aa2b4db7a0449a7bb030d70cdc3780fc59cafddf6ff071beb36365b44e2d</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>56</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>https://github.com/SemiAnalysisAI/InferenceX-app/releases/download/db-dump/2026-05-11/inferencex-dump-2026-05-11.zip</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>https://github.com/SemiAnalysisAI/InferenceX-app/releases/tag/db-dump/2026-05-11</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>Weekly database dump.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>SemiAnalysisAI/InferenceX-app</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>db-dump/2026-05-04</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>DB Dump 2026-05-04</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>2026-05-04T01:02:14Z</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>inferencex-dump-2026-05-04.zip</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>1696315703</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>sha256:855534ca7b6b4ef4281b60641f9f7089f8369b14c93024d3b7f1f73cb2050c94</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>58</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>https://github.com/SemiAnalysisAI/InferenceX-app/releases/download/db-dump/2026-05-04/inferencex-dump-2026-05-04.zip</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>https://github.com/SemiAnalysisAI/InferenceX-app/releases/tag/db-dump/2026-05-04</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>Weekly database dump.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>SemiAnalysisAI/InferenceX-app</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>db-dump/2026-04-27</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>DB Dump 2026-04-27</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-27T00:47:55Z</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>inferencex-dump-2026-04-27.zip</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>258632807</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>sha256:3f31c5c30e19e8e317329dea81e974b0dae563f25bc4be7f92dea11defa9100c</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>73</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>https://github.com/SemiAnalysisAI/InferenceX-app/releases/download/db-dump/2026-04-27/inferencex-dump-2026-04-27.zip</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>https://github.com/SemiAnalysisAI/InferenceX-app/releases/tag/db-dump/2026-04-27</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>Weekly database dump.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>SemiAnalysisAI/InferenceX-app</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>db-dump/2026-04-20</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>DB Dump 2026-04-20</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-20T00:45:46Z</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>inferencex-dump-2026-04-20.zip</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>241981257</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>sha256:4d0dced5e75861d8fb4e66ac8c023270fb8f0eb2c321704f0aeff47de5d4499d</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>43</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>https://github.com/SemiAnalysisAI/InferenceX-app/releases/download/db-dump/2026-04-20/inferencex-dump-2026-04-20.zip</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>https://github.com/SemiAnalysisAI/InferenceX-app/releases/tag/db-dump/2026-04-20</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>Weekly database dump.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>SemiAnalysisAI/InferenceX-app</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>db-dump/2026-04-13</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>DB Dump 2026-04-13</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-13T00:46:55Z</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>inferencex-dump-2026-04-13.zip</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>209158762</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>sha256:bd64a9b291a65078556572907afe290e8cab150b69bd90e3e83d6c84bb07e472</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>https://github.com/SemiAnalysisAI/InferenceX-app/releases/download/db-dump/2026-04-13/inferencex-dump-2026-04-13.zip</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>https://github.com/SemiAnalysisAI/InferenceX-app/releases/tag/db-dump/2026-04-13</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>Weekly database dump.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>SemiAnalysisAI/InferenceX-app</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>db-dump/2026-04-06</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>DB Dump 2026-04-06</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>2026-04-06T00:42:05Z</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>inferencex-dump-2026-04-06.zip</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>199263597</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>sha256:f95a724b6eeba403456fb8b87a2283e86e41a7f055f4e2dedbd81a3c8462c37c</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>https://github.com/SemiAnalysisAI/InferenceX-app/releases/download/db-dump/2026-04-06/inferencex-dump-2026-04-06.zip</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>https://github.com/SemiAnalysisAI/InferenceX-app/releases/tag/db-dump/2026-04-06</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>Weekly database dump.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>SemiAnalysisAI/InferenceX-app</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>db-dump/2026-03-30</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>DB Dump 2026-03-30</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-30T00:42:36Z</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>inferencex-dump-2026-03-30.zip</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>177537481</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>sha256:20a5d7ad79659afbe12af37074067cf8655f52bec68e034675612b5845033587</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>109</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>https://github.com/SemiAnalysisAI/InferenceX-app/releases/download/db-dump/2026-03-30/inferencex-dump-2026-03-30.zip</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>https://github.com/SemiAnalysisAI/InferenceX-app/releases/tag/db-dump/2026-03-30</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>Weekly database dump.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>SemiAnalysisAI/InferenceX-app</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>db-dump/2026-03-28</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>DB Dump 2026-03-28</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>2026-03-28T06:04:13Z</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>inferencex-dump-2026-03-28.zip</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>187401353</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>sha256:d5697c68864346875548d7891ee77addf7559aba111d6710c28325352409e6f7</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>https://github.com/SemiAnalysisAI/InferenceX-app/releases/download/db-dump/2026-03-28/inferencex-dump-2026-03-28.zip</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>https://github.com/SemiAnalysisAI/InferenceX-app/releases/tag/db-dump/2026-03-28</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>Weekly database dump.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:K9"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:H16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="29" customWidth="1" min="2" max="2"/>
+    <col width="38" customWidth="1" min="3" max="3"/>
+    <col width="38" customWidth="1" min="4" max="4"/>
+    <col width="38" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="38" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>check_id</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>area</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>question_kr</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>pass_criteria_kr</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>risk_if_fail_kr</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>owner</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>severity</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>current_status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>HC01</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Source existence</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>모든 source URL 또는 report name이 실제로 존재하고 접근 가능한가?</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>01_sources의 URL을 열었을 때 publisher/title/date가 일치한다.</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>없는 출처 또는 잘못된 출처를 근거로 사용.</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>Research</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>Needs manual URL click-through</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>HC02</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Numeric fact quote</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>Fact anchor의 숫자(예: 4.5GW, 671B/37B, 235B/22B, 100k GPU)가 원문에 직접 존재하는가?</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>02a_fact_anchors의 value가 원문 문장/표와 직접 매칭된다.</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>proxy나 추정을 fact처럼 표시.</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>Research</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>Partially checked; requires final source screenshot/quote pack</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>HC03</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Fact vs estimate separation</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>Active GW, inference share, utilization, tokens/sec/MW가 fact로 오표기되지 않았는가?</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>해당 값은 Estimate/Scenario로 표시되고 replacement_path가 있다.</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>임원 보고에서 확정 수치처럼 오해.</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>Model</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>Pass in structure</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>HC04</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Closed model parameters</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>OpenAI, Anthropic, Gemini, Grok 같은 closed model에 단일 precise parameter 숫자를 쓰지 않았는가?</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>closed model은 band/proxy로만 표시하고 benchmark는 sanity check로만 사용.</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>비공개 파라미터 hallucination.</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>Model</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>HC05</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>MoE total/active</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>MoE 모델은 total params와 active params를 분리했는가?</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>DeepSeek, Qwen, Llama 4 계열은 total/active가 별도 column 또는 anchor에 존재.</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>MoE 효율을 과소/과대 계산.</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>Model</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>HC06</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Host vs model owner</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>AWS/Google/Oracle 같은 host capacity가 model owner와 혼동되지 않았는가?</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Anthropic/OpenAI capacity는 model output 기준으로 귀속하고 host는 source/context로만 표기.</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>capacity double count 또는 wrong attribution.</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>Model</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>Pass in attribution rules</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>HC07</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Microsoft/OpenAI overlap</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>Microsoft Copilot token과 OpenAI model token을 이중계산하지 않았는가?</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>OpenAI model output은 OpenAI row, Microsoft-owned/serving burden은 Microsoft row로 명시.</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>OpenAI/Microsoft capacity 중복 산정.</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>Model</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>Needs sales/product routing data for final resolution</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>HC08</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Capacity boundary</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>active_power_gw가 contracted_power_gw를 넘지 않는가?</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>모든 company-year-scenario에서 active &lt;= contracted.</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>물리적으로 불가능한 deployment.</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>Model</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>Automated pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>HC09</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Power split</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>training_power_share + inference_power_share = 100%인가?</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>모든 row에서 합계가 1.000 +/- 0.001.</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>GW가 누락 또는 중복.</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>Model</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>Automated pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>HC10</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Unit consistency</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>daily token과 annual token 단위가 섞이지 않았는가?</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>token/day는 86,400초, annual token은 365일 또는 31,536,000초로 환산.</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>365배 오류 또는 daily/annual 비교 오류.</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>Model</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>Automated pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>HC11</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Benchmark proxy use</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>OSS/open benchmark를 closed commercial model 결론으로 직접 사용하지 않았는가?</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>08d_benchmark_reference는 sanity check이며 main forecast와 분리.</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>gpt-oss/Qwen/Llama benchmark를 GPT/Claude/Gemini 실서비스로 오인.</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>Model</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>HC12</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Inference share</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>2026년 추론 60%+를 fact로 단정하지 않았는가?</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>Base 2026은 60% 미만이고 Bull에서만 60%+ 허용.</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>전망을 현재 fact처럼 보고.</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>Model</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>HC13</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Outlier review</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>main forecast와 benchmark reference의 차이가 큰 업체를 따로 표시했는가?</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>benchmark_vs_model_pct가 +/-50%를 넘으면 confidence review 대상.</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>과감한 가정을 숨긴 채 보고.</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>Model</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>Needs reviewer sign-off</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>HC14</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>China transparency</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>중국 업체의 낮은 공개성 때문에 수치를 임의로 페널티하거나 과신하지 않았는가?</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>모델 구조 fact는 인정하고 capacity transparency만 confidence에 반영.</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>bias 또는 confidence mislabeling.</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>Research</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>Pass in principle; needs Chinese primary-source review</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>HC15</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>Executive wording</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>슬라이드 문구가 추정치를 확정 사실처럼 표현하지 않는가?</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>forecast, scenario, proxy, sanity check, 추정치 표현을 유지.</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>의사결정자가 불확실성을 과소평가.</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>Presentation</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>Needs final human review</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:H16"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet23.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="38" customWidth="1" min="1" max="1"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="29" customWidth="1" min="3" max="3"/>
+    <col width="38" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>metric</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>value</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>display</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>interpretation_kr</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>2030 core-company inference tokens/day</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="n">
+        <v>2871987625721952</v>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>2.87 quadrillion tokens/day</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>9개 상용 LLM owner의 base case 총 생성 capacity.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>2030 inference AI IT load</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="n">
+        <v>23.02</v>
+      </c>
+      <c r="C3" s="2" t="inlineStr">
+        <is>
+          <t>23.02 GW inference load</t>
+        </is>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>PUE와 AI workload share 차감 후 inference에 배정된 IT load.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>2030 US vs China split</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr"/>
+      <c r="C4" s="2" t="inlineStr">
+        <is>
+          <t>US 81% / China 19%</t>
+        </is>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>회사 owner 기준 split이며 AWS/Oracle/CoreWeave 같은 host는 core row가 아님.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Rank 1: OpenAI 2030 tokens/day</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>586840240711296</v>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>0.59Q/day</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>GPT / o-series / ChatGPT serving capacity; confidence=Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Rank 2: Google 2030 tokens/day</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="n">
+        <v>535132862530560</v>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>0.54Q/day</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>Gemini / Gemma serving capacity; confidence=Medium-High</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Rank 3: Meta 2030 tokens/day</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="n">
+        <v>402286619750400</v>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>0.40Q/day</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>Llama / Meta AI serving capacity; confidence=Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Rank 4: Microsoft 2030 tokens/day</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="n">
+        <v>372288096107136</v>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>0.37Q/day</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>Phi / MAI / Copilot model mix serving capacity; confidence=Medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Rank 5: Anthropic 2030 tokens/day</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="n">
+        <v>318303245151360</v>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>0.32Q/day</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>Claude Opus / Sonnet / Haiku serving capacity; confidence=Medium</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:D9"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet24.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Expand Excel output to token time series
</commit_message>
<xml_diff>
--- a/llm_token_capacity_project/outputs/reports/llm_token_capacity_2026_2030.xlsx
+++ b/llm_token_capacity_project/outputs/reports/llm_token_capacity_2026_2030.xlsx
@@ -33,7 +33,7 @@
     <numFmt numFmtId="164" formatCode="0.0%"/>
     <numFmt numFmtId="165" formatCode="0.000"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -59,10 +59,15 @@
     </font>
     <font>
       <b val="1"/>
+      <color rgb="0014213D"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <b val="1"/>
       <color rgb="00006100"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -89,6 +94,11 @@
         <fgColor rgb="00E2F0D9"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9EAF7"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="2">
     <border>
@@ -107,7 +117,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -141,16 +151,22 @@
     <xf numFmtId="3" fontId="0" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="165" fontId="2" fillId="6" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -243,7 +259,7 @@
               <a:defRPr/>
             </a:pPr>
             <a:r>
-              <a:t>Scenario Token Capacity (Q tokens/day)</a:t>
+              <a:t>Base Provider Token Capacity (Q tokens/day)</a:t>
             </a:r>
           </a:p>
         </rich>
@@ -256,9 +272,7 @@
           <idx val="0"/>
           <order val="0"/>
           <tx>
-            <strRef>
-              <f>'04_Output'!B12</f>
-            </strRef>
+            <v>Microsoft</v>
           </tx>
           <spPr>
             <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
@@ -275,12 +289,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'04_Output'!$A$13:$A$17</f>
+              <f>'04_Output'!$B$5:$F$5</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'04_Output'!$B$13:$B$17</f>
+              <f>'04_Output'!$B$6:$F$6</f>
             </numRef>
           </val>
         </ser>
@@ -288,9 +302,7 @@
           <idx val="1"/>
           <order val="1"/>
           <tx>
-            <strRef>
-              <f>'04_Output'!C12</f>
-            </strRef>
+            <v>Google</v>
           </tx>
           <spPr>
             <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
@@ -307,12 +319,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'04_Output'!$A$13:$A$17</f>
+              <f>'04_Output'!$B$5:$F$5</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'04_Output'!$C$13:$C$17</f>
+              <f>'04_Output'!$B$7:$F$7</f>
             </numRef>
           </val>
         </ser>
@@ -320,9 +332,7 @@
           <idx val="2"/>
           <order val="2"/>
           <tx>
-            <strRef>
-              <f>'04_Output'!D12</f>
-            </strRef>
+            <v>Meta</v>
           </tx>
           <spPr>
             <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
@@ -339,12 +349,12 @@
           </marker>
           <cat>
             <numRef>
-              <f>'04_Output'!$A$13:$A$17</f>
+              <f>'04_Output'!$B$5:$F$5</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'04_Output'!$D$13:$D$17</f>
+              <f>'04_Output'!$B$8:$F$8</f>
             </numRef>
           </val>
         </ser>
@@ -352,9 +362,7 @@
           <idx val="3"/>
           <order val="3"/>
           <tx>
-            <strRef>
-              <f>'04_Output'!E12</f>
-            </strRef>
+            <v>xAI</v>
           </tx>
           <spPr>
             <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
@@ -371,12 +379,162 @@
           </marker>
           <cat>
             <numRef>
-              <f>'04_Output'!$A$13:$A$17</f>
+              <f>'04_Output'!$B$5:$F$5</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'04_Output'!$E$13:$E$17</f>
+              <f>'04_Output'!$B$9:$F$9</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="4"/>
+          <order val="4"/>
+          <tx>
+            <v>OpenAI</v>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'04_Output'!$B$5:$F$5</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'04_Output'!$B$10:$F$10</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="5"/>
+          <order val="5"/>
+          <tx>
+            <v>Anthropic</v>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'04_Output'!$B$5:$F$5</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'04_Output'!$B$11:$F$11</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="6"/>
+          <order val="6"/>
+          <tx>
+            <v>DeepSeek</v>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'04_Output'!$B$5:$F$5</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'04_Output'!$B$12:$F$12</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="7"/>
+          <order val="7"/>
+          <tx>
+            <v>Alibaba</v>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'04_Output'!$B$5:$F$5</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'04_Output'!$B$13:$F$13</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="8"/>
+          <order val="8"/>
+          <tx>
+            <v>Tencent</v>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'04_Output'!$B$5:$F$5</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'04_Output'!$B$14:$F$14</f>
             </numRef>
           </val>
         </ser>
@@ -431,6 +589,7 @@
             </rich>
           </tx>
         </title>
+        <numFmt formatCode="0.000" sourceLinked="0"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="10"/>
@@ -446,6 +605,213 @@
 </file>
 
 <file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Scenario Total Token Capacity (Q tokens/day)</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <v>Bear</v>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'04_Output'!$B$31:$F$31</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'04_Output'!$B$32:$F$32</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <v>Base</v>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'04_Output'!$B$31:$F$31</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'04_Output'!$B$33:$F$33</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="2"/>
+          <order val="2"/>
+          <tx>
+            <v>Bull</v>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'04_Output'!$B$31:$F$31</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'04_Output'!$B$34:$F$34</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="3"/>
+          <order val="3"/>
+          <tx>
+            <v>Grid-Constrained / Efficiency-Upside</v>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'04_Output'!$B$31:$F$31</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'04_Output'!$B$35:$F$35</f>
+            </numRef>
+          </val>
+        </ser>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Year</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <title>
+          <tx>
+            <rich>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:pPr>
+                  <a:defRPr/>
+                </a:pPr>
+                <a:r>
+                  <a:t>Q tokens/day</a:t>
+                </a:r>
+              </a:p>
+            </rich>
+          </tx>
+        </title>
+        <numFmt formatCode="0.000" sourceLinked="0"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart3.xml><?xml version="1.0" encoding="utf-8"?>
 <chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
@@ -631,9 +997,9 @@
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
-      <col>8</col>
+      <col>7</col>
       <colOff>0</colOff>
-      <row>1</row>
+      <row>3</row>
       <rowOff>0</rowOff>
     </from>
     <ext cx="6480000" cy="2880000"/>
@@ -646,6 +1012,28 @@
       <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
           <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>7</col>
+      <colOff>0</colOff>
+      <row>21</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="6480000" cy="2880000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="2" name="Chart 2"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -34249,488 +34637,959 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G18"/>
+  <dimension ref="A1:F42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="27" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="21" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="21" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="46" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Base Scenario: Generated Output Token Capacity</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="13" t="inlineStr">
+          <t>Base Scenario: Generated Output Token Capacity, 2026-2030</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="34" customHeight="1">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>업체별 output은 Base scenario 기준이며, 모든 수치는 `03_Calculation`의 generated output token formula를 직접 참조합니다. 단위는 Quadrillion (Q) tokens입니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="n"/>
+      <c r="B3" s="3" t="n"/>
+      <c r="C3" s="3" t="n"/>
+      <c r="D3" s="3" t="n"/>
+      <c r="E3" s="3" t="n"/>
+      <c r="F3" s="3" t="n"/>
+    </row>
+    <row r="4">
+      <c r="A4" s="13" t="inlineStr">
+        <is>
+          <t>Base Provider Time Series - Generated Output Tokens/Day (Q)</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="n"/>
+      <c r="C4" s="3" t="n"/>
+      <c r="D4" s="3" t="n"/>
+      <c r="E4" s="3" t="n"/>
+      <c r="F4" s="3" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="14" t="inlineStr">
         <is>
           <t>Provider</t>
         </is>
       </c>
-      <c r="B2" s="13" t="inlineStr">
-        <is>
-          <t>Year</t>
-        </is>
-      </c>
-      <c r="C2" s="13" t="inlineStr">
-        <is>
-          <t>Operational GW</t>
-        </is>
-      </c>
-      <c r="D2" s="13" t="inlineStr">
-        <is>
-          <t>Inference GW</t>
-        </is>
-      </c>
-      <c r="E2" s="13" t="inlineStr">
-        <is>
-          <t>Selected TPS/MW</t>
-        </is>
-      </c>
-      <c r="F2" s="13" t="inlineStr">
-        <is>
-          <t>Tokens/Day (Q)</t>
-        </is>
-      </c>
-      <c r="G2" s="13" t="inlineStr">
-        <is>
-          <t>Tokens/Year (Q)</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="9">
-        <f>'03_Calculation'!B51</f>
-        <v/>
-      </c>
-      <c r="B3" s="9">
-        <f>'03_Calculation'!C51</f>
-        <v/>
-      </c>
-      <c r="C3" s="11">
-        <f>'03_Calculation'!F51</f>
-        <v/>
-      </c>
-      <c r="D3" s="11">
-        <f>'03_Calculation'!L51</f>
-        <v/>
-      </c>
-      <c r="E3" s="9">
-        <f>'03_Calculation'!X51</f>
-        <v/>
-      </c>
-      <c r="F3" s="11">
-        <f>'03_Calculation'!Y51/1000000000000000</f>
-        <v/>
-      </c>
-      <c r="G3" s="11">
-        <f>'03_Calculation'!Z51/1000000000000000</f>
-        <v/>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="9">
-        <f>'03_Calculation'!B56</f>
-        <v/>
-      </c>
-      <c r="B4" s="9">
-        <f>'03_Calculation'!C56</f>
-        <v/>
-      </c>
-      <c r="C4" s="11">
-        <f>'03_Calculation'!F56</f>
-        <v/>
-      </c>
-      <c r="D4" s="11">
-        <f>'03_Calculation'!L56</f>
-        <v/>
-      </c>
-      <c r="E4" s="9">
-        <f>'03_Calculation'!X56</f>
-        <v/>
-      </c>
-      <c r="F4" s="11">
-        <f>'03_Calculation'!Y56/1000000000000000</f>
-        <v/>
-      </c>
-      <c r="G4" s="11">
-        <f>'03_Calculation'!Z56/1000000000000000</f>
-        <v/>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="9">
-        <f>'03_Calculation'!B61</f>
-        <v/>
-      </c>
-      <c r="B5" s="9">
-        <f>'03_Calculation'!C61</f>
-        <v/>
-      </c>
-      <c r="C5" s="11">
-        <f>'03_Calculation'!F61</f>
-        <v/>
-      </c>
-      <c r="D5" s="11">
-        <f>'03_Calculation'!L61</f>
-        <v/>
-      </c>
-      <c r="E5" s="9">
-        <f>'03_Calculation'!X61</f>
-        <v/>
-      </c>
-      <c r="F5" s="11">
-        <f>'03_Calculation'!Y61/1000000000000000</f>
-        <v/>
-      </c>
-      <c r="G5" s="11">
-        <f>'03_Calculation'!Z61/1000000000000000</f>
-        <v/>
+      <c r="B5" s="14" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C5" s="14" t="n">
+        <v>2027</v>
+      </c>
+      <c r="D5" s="14" t="n">
+        <v>2028</v>
+      </c>
+      <c r="E5" s="14" t="n">
+        <v>2029</v>
+      </c>
+      <c r="F5" s="14" t="n">
+        <v>2030</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="9">
-        <f>'03_Calculation'!B66</f>
-        <v/>
-      </c>
-      <c r="B6" s="9">
-        <f>'03_Calculation'!C66</f>
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Microsoft</t>
+        </is>
+      </c>
+      <c r="B6" s="11">
+        <f>SUMIFS('03_Calculation'!$Y$2:$Y$181,'03_Calculation'!$A$2:$A$181,"Base",'03_Calculation'!$B$2:$B$181,$A6,'03_Calculation'!$C$2:$C$181,B$5)/1000000000000000</f>
         <v/>
       </c>
       <c r="C6" s="11">
-        <f>'03_Calculation'!F66</f>
+        <f>SUMIFS('03_Calculation'!$Y$2:$Y$181,'03_Calculation'!$A$2:$A$181,"Base",'03_Calculation'!$B$2:$B$181,$A6,'03_Calculation'!$C$2:$C$181,C$5)/1000000000000000</f>
         <v/>
       </c>
       <c r="D6" s="11">
-        <f>'03_Calculation'!L66</f>
-        <v/>
-      </c>
-      <c r="E6" s="9">
-        <f>'03_Calculation'!X66</f>
+        <f>SUMIFS('03_Calculation'!$Y$2:$Y$181,'03_Calculation'!$A$2:$A$181,"Base",'03_Calculation'!$B$2:$B$181,$A6,'03_Calculation'!$C$2:$C$181,D$5)/1000000000000000</f>
+        <v/>
+      </c>
+      <c r="E6" s="11">
+        <f>SUMIFS('03_Calculation'!$Y$2:$Y$181,'03_Calculation'!$A$2:$A$181,"Base",'03_Calculation'!$B$2:$B$181,$A6,'03_Calculation'!$C$2:$C$181,E$5)/1000000000000000</f>
         <v/>
       </c>
       <c r="F6" s="11">
-        <f>'03_Calculation'!Y66/1000000000000000</f>
-        <v/>
-      </c>
-      <c r="G6" s="11">
-        <f>'03_Calculation'!Z66/1000000000000000</f>
+        <f>SUMIFS('03_Calculation'!$Y$2:$Y$181,'03_Calculation'!$A$2:$A$181,"Base",'03_Calculation'!$B$2:$B$181,$A6,'03_Calculation'!$C$2:$C$181,F$5)/1000000000000000</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="9">
-        <f>'03_Calculation'!B71</f>
-        <v/>
-      </c>
-      <c r="B7" s="9">
-        <f>'03_Calculation'!C71</f>
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Google</t>
+        </is>
+      </c>
+      <c r="B7" s="11">
+        <f>SUMIFS('03_Calculation'!$Y$2:$Y$181,'03_Calculation'!$A$2:$A$181,"Base",'03_Calculation'!$B$2:$B$181,$A7,'03_Calculation'!$C$2:$C$181,B$5)/1000000000000000</f>
         <v/>
       </c>
       <c r="C7" s="11">
-        <f>'03_Calculation'!F71</f>
+        <f>SUMIFS('03_Calculation'!$Y$2:$Y$181,'03_Calculation'!$A$2:$A$181,"Base",'03_Calculation'!$B$2:$B$181,$A7,'03_Calculation'!$C$2:$C$181,C$5)/1000000000000000</f>
         <v/>
       </c>
       <c r="D7" s="11">
-        <f>'03_Calculation'!L71</f>
-        <v/>
-      </c>
-      <c r="E7" s="9">
-        <f>'03_Calculation'!X71</f>
+        <f>SUMIFS('03_Calculation'!$Y$2:$Y$181,'03_Calculation'!$A$2:$A$181,"Base",'03_Calculation'!$B$2:$B$181,$A7,'03_Calculation'!$C$2:$C$181,D$5)/1000000000000000</f>
+        <v/>
+      </c>
+      <c r="E7" s="11">
+        <f>SUMIFS('03_Calculation'!$Y$2:$Y$181,'03_Calculation'!$A$2:$A$181,"Base",'03_Calculation'!$B$2:$B$181,$A7,'03_Calculation'!$C$2:$C$181,E$5)/1000000000000000</f>
         <v/>
       </c>
       <c r="F7" s="11">
-        <f>'03_Calculation'!Y71/1000000000000000</f>
-        <v/>
-      </c>
-      <c r="G7" s="11">
-        <f>'03_Calculation'!Z71/1000000000000000</f>
+        <f>SUMIFS('03_Calculation'!$Y$2:$Y$181,'03_Calculation'!$A$2:$A$181,"Base",'03_Calculation'!$B$2:$B$181,$A7,'03_Calculation'!$C$2:$C$181,F$5)/1000000000000000</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="9">
-        <f>'03_Calculation'!B76</f>
-        <v/>
-      </c>
-      <c r="B8" s="9">
-        <f>'03_Calculation'!C76</f>
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>Meta</t>
+        </is>
+      </c>
+      <c r="B8" s="11">
+        <f>SUMIFS('03_Calculation'!$Y$2:$Y$181,'03_Calculation'!$A$2:$A$181,"Base",'03_Calculation'!$B$2:$B$181,$A8,'03_Calculation'!$C$2:$C$181,B$5)/1000000000000000</f>
         <v/>
       </c>
       <c r="C8" s="11">
-        <f>'03_Calculation'!F76</f>
+        <f>SUMIFS('03_Calculation'!$Y$2:$Y$181,'03_Calculation'!$A$2:$A$181,"Base",'03_Calculation'!$B$2:$B$181,$A8,'03_Calculation'!$C$2:$C$181,C$5)/1000000000000000</f>
         <v/>
       </c>
       <c r="D8" s="11">
-        <f>'03_Calculation'!L76</f>
-        <v/>
-      </c>
-      <c r="E8" s="9">
-        <f>'03_Calculation'!X76</f>
+        <f>SUMIFS('03_Calculation'!$Y$2:$Y$181,'03_Calculation'!$A$2:$A$181,"Base",'03_Calculation'!$B$2:$B$181,$A8,'03_Calculation'!$C$2:$C$181,D$5)/1000000000000000</f>
+        <v/>
+      </c>
+      <c r="E8" s="11">
+        <f>SUMIFS('03_Calculation'!$Y$2:$Y$181,'03_Calculation'!$A$2:$A$181,"Base",'03_Calculation'!$B$2:$B$181,$A8,'03_Calculation'!$C$2:$C$181,E$5)/1000000000000000</f>
         <v/>
       </c>
       <c r="F8" s="11">
-        <f>'03_Calculation'!Y76/1000000000000000</f>
-        <v/>
-      </c>
-      <c r="G8" s="11">
-        <f>'03_Calculation'!Z76/1000000000000000</f>
+        <f>SUMIFS('03_Calculation'!$Y$2:$Y$181,'03_Calculation'!$A$2:$A$181,"Base",'03_Calculation'!$B$2:$B$181,$A8,'03_Calculation'!$C$2:$C$181,F$5)/1000000000000000</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="9">
-        <f>'03_Calculation'!B81</f>
-        <v/>
-      </c>
-      <c r="B9" s="9">
-        <f>'03_Calculation'!C81</f>
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>xAI</t>
+        </is>
+      </c>
+      <c r="B9" s="11">
+        <f>SUMIFS('03_Calculation'!$Y$2:$Y$181,'03_Calculation'!$A$2:$A$181,"Base",'03_Calculation'!$B$2:$B$181,$A9,'03_Calculation'!$C$2:$C$181,B$5)/1000000000000000</f>
         <v/>
       </c>
       <c r="C9" s="11">
-        <f>'03_Calculation'!F81</f>
+        <f>SUMIFS('03_Calculation'!$Y$2:$Y$181,'03_Calculation'!$A$2:$A$181,"Base",'03_Calculation'!$B$2:$B$181,$A9,'03_Calculation'!$C$2:$C$181,C$5)/1000000000000000</f>
         <v/>
       </c>
       <c r="D9" s="11">
-        <f>'03_Calculation'!L81</f>
-        <v/>
-      </c>
-      <c r="E9" s="9">
-        <f>'03_Calculation'!X81</f>
+        <f>SUMIFS('03_Calculation'!$Y$2:$Y$181,'03_Calculation'!$A$2:$A$181,"Base",'03_Calculation'!$B$2:$B$181,$A9,'03_Calculation'!$C$2:$C$181,D$5)/1000000000000000</f>
+        <v/>
+      </c>
+      <c r="E9" s="11">
+        <f>SUMIFS('03_Calculation'!$Y$2:$Y$181,'03_Calculation'!$A$2:$A$181,"Base",'03_Calculation'!$B$2:$B$181,$A9,'03_Calculation'!$C$2:$C$181,E$5)/1000000000000000</f>
         <v/>
       </c>
       <c r="F9" s="11">
-        <f>'03_Calculation'!Y81/1000000000000000</f>
-        <v/>
-      </c>
-      <c r="G9" s="11">
-        <f>'03_Calculation'!Z81/1000000000000000</f>
+        <f>SUMIFS('03_Calculation'!$Y$2:$Y$181,'03_Calculation'!$A$2:$A$181,"Base",'03_Calculation'!$B$2:$B$181,$A9,'03_Calculation'!$C$2:$C$181,F$5)/1000000000000000</f>
         <v/>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="9">
-        <f>'03_Calculation'!B86</f>
-        <v/>
-      </c>
-      <c r="B10" s="9">
-        <f>'03_Calculation'!C86</f>
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="B10" s="11">
+        <f>SUMIFS('03_Calculation'!$Y$2:$Y$181,'03_Calculation'!$A$2:$A$181,"Base",'03_Calculation'!$B$2:$B$181,$A10,'03_Calculation'!$C$2:$C$181,B$5)/1000000000000000</f>
         <v/>
       </c>
       <c r="C10" s="11">
-        <f>'03_Calculation'!F86</f>
+        <f>SUMIFS('03_Calculation'!$Y$2:$Y$181,'03_Calculation'!$A$2:$A$181,"Base",'03_Calculation'!$B$2:$B$181,$A10,'03_Calculation'!$C$2:$C$181,C$5)/1000000000000000</f>
         <v/>
       </c>
       <c r="D10" s="11">
-        <f>'03_Calculation'!L86</f>
-        <v/>
-      </c>
-      <c r="E10" s="9">
-        <f>'03_Calculation'!X86</f>
+        <f>SUMIFS('03_Calculation'!$Y$2:$Y$181,'03_Calculation'!$A$2:$A$181,"Base",'03_Calculation'!$B$2:$B$181,$A10,'03_Calculation'!$C$2:$C$181,D$5)/1000000000000000</f>
+        <v/>
+      </c>
+      <c r="E10" s="11">
+        <f>SUMIFS('03_Calculation'!$Y$2:$Y$181,'03_Calculation'!$A$2:$A$181,"Base",'03_Calculation'!$B$2:$B$181,$A10,'03_Calculation'!$C$2:$C$181,E$5)/1000000000000000</f>
         <v/>
       </c>
       <c r="F10" s="11">
-        <f>'03_Calculation'!Y86/1000000000000000</f>
-        <v/>
-      </c>
-      <c r="G10" s="11">
-        <f>'03_Calculation'!Z86/1000000000000000</f>
+        <f>SUMIFS('03_Calculation'!$Y$2:$Y$181,'03_Calculation'!$A$2:$A$181,"Base",'03_Calculation'!$B$2:$B$181,$A10,'03_Calculation'!$C$2:$C$181,F$5)/1000000000000000</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="9">
-        <f>'03_Calculation'!B91</f>
-        <v/>
-      </c>
-      <c r="B11" s="9">
-        <f>'03_Calculation'!C91</f>
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>Anthropic</t>
+        </is>
+      </c>
+      <c r="B11" s="11">
+        <f>SUMIFS('03_Calculation'!$Y$2:$Y$181,'03_Calculation'!$A$2:$A$181,"Base",'03_Calculation'!$B$2:$B$181,$A11,'03_Calculation'!$C$2:$C$181,B$5)/1000000000000000</f>
         <v/>
       </c>
       <c r="C11" s="11">
-        <f>'03_Calculation'!F91</f>
+        <f>SUMIFS('03_Calculation'!$Y$2:$Y$181,'03_Calculation'!$A$2:$A$181,"Base",'03_Calculation'!$B$2:$B$181,$A11,'03_Calculation'!$C$2:$C$181,C$5)/1000000000000000</f>
         <v/>
       </c>
       <c r="D11" s="11">
-        <f>'03_Calculation'!L91</f>
-        <v/>
-      </c>
-      <c r="E11" s="9">
-        <f>'03_Calculation'!X91</f>
+        <f>SUMIFS('03_Calculation'!$Y$2:$Y$181,'03_Calculation'!$A$2:$A$181,"Base",'03_Calculation'!$B$2:$B$181,$A11,'03_Calculation'!$C$2:$C$181,D$5)/1000000000000000</f>
+        <v/>
+      </c>
+      <c r="E11" s="11">
+        <f>SUMIFS('03_Calculation'!$Y$2:$Y$181,'03_Calculation'!$A$2:$A$181,"Base",'03_Calculation'!$B$2:$B$181,$A11,'03_Calculation'!$C$2:$C$181,E$5)/1000000000000000</f>
         <v/>
       </c>
       <c r="F11" s="11">
-        <f>'03_Calculation'!Y91/1000000000000000</f>
-        <v/>
-      </c>
-      <c r="G11" s="11">
-        <f>'03_Calculation'!Z91/1000000000000000</f>
+        <f>SUMIFS('03_Calculation'!$Y$2:$Y$181,'03_Calculation'!$A$2:$A$181,"Base",'03_Calculation'!$B$2:$B$181,$A11,'03_Calculation'!$C$2:$C$181,F$5)/1000000000000000</f>
         <v/>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="14" t="n"/>
-      <c r="B12" s="14" t="n"/>
-      <c r="C12" s="14" t="n"/>
-      <c r="D12" s="14" t="n"/>
-      <c r="E12" s="14" t="n"/>
-      <c r="F12" s="14" t="n"/>
-      <c r="G12" s="14" t="n"/>
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>DeepSeek</t>
+        </is>
+      </c>
+      <c r="B12" s="11">
+        <f>SUMIFS('03_Calculation'!$Y$2:$Y$181,'03_Calculation'!$A$2:$A$181,"Base",'03_Calculation'!$B$2:$B$181,$A12,'03_Calculation'!$C$2:$C$181,B$5)/1000000000000000</f>
+        <v/>
+      </c>
+      <c r="C12" s="11">
+        <f>SUMIFS('03_Calculation'!$Y$2:$Y$181,'03_Calculation'!$A$2:$A$181,"Base",'03_Calculation'!$B$2:$B$181,$A12,'03_Calculation'!$C$2:$C$181,C$5)/1000000000000000</f>
+        <v/>
+      </c>
+      <c r="D12" s="11">
+        <f>SUMIFS('03_Calculation'!$Y$2:$Y$181,'03_Calculation'!$A$2:$A$181,"Base",'03_Calculation'!$B$2:$B$181,$A12,'03_Calculation'!$C$2:$C$181,D$5)/1000000000000000</f>
+        <v/>
+      </c>
+      <c r="E12" s="11">
+        <f>SUMIFS('03_Calculation'!$Y$2:$Y$181,'03_Calculation'!$A$2:$A$181,"Base",'03_Calculation'!$B$2:$B$181,$A12,'03_Calculation'!$C$2:$C$181,E$5)/1000000000000000</f>
+        <v/>
+      </c>
+      <c r="F12" s="11">
+        <f>SUMIFS('03_Calculation'!$Y$2:$Y$181,'03_Calculation'!$A$2:$A$181,"Base",'03_Calculation'!$B$2:$B$181,$A12,'03_Calculation'!$C$2:$C$181,F$5)/1000000000000000</f>
+        <v/>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="3" t="inlineStr">
         <is>
-          <t>Scenario Time Series (Q generated output tokens/day)</t>
-        </is>
-      </c>
-      <c r="B13" s="15" t="inlineStr">
+          <t>Alibaba</t>
+        </is>
+      </c>
+      <c r="B13" s="11">
+        <f>SUMIFS('03_Calculation'!$Y$2:$Y$181,'03_Calculation'!$A$2:$A$181,"Base",'03_Calculation'!$B$2:$B$181,$A13,'03_Calculation'!$C$2:$C$181,B$5)/1000000000000000</f>
+        <v/>
+      </c>
+      <c r="C13" s="11">
+        <f>SUMIFS('03_Calculation'!$Y$2:$Y$181,'03_Calculation'!$A$2:$A$181,"Base",'03_Calculation'!$B$2:$B$181,$A13,'03_Calculation'!$C$2:$C$181,C$5)/1000000000000000</f>
+        <v/>
+      </c>
+      <c r="D13" s="11">
+        <f>SUMIFS('03_Calculation'!$Y$2:$Y$181,'03_Calculation'!$A$2:$A$181,"Base",'03_Calculation'!$B$2:$B$181,$A13,'03_Calculation'!$C$2:$C$181,D$5)/1000000000000000</f>
+        <v/>
+      </c>
+      <c r="E13" s="11">
+        <f>SUMIFS('03_Calculation'!$Y$2:$Y$181,'03_Calculation'!$A$2:$A$181,"Base",'03_Calculation'!$B$2:$B$181,$A13,'03_Calculation'!$C$2:$C$181,E$5)/1000000000000000</f>
+        <v/>
+      </c>
+      <c r="F13" s="11">
+        <f>SUMIFS('03_Calculation'!$Y$2:$Y$181,'03_Calculation'!$A$2:$A$181,"Base",'03_Calculation'!$B$2:$B$181,$A13,'03_Calculation'!$C$2:$C$181,F$5)/1000000000000000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>Tencent</t>
+        </is>
+      </c>
+      <c r="B14" s="11">
+        <f>SUMIFS('03_Calculation'!$Y$2:$Y$181,'03_Calculation'!$A$2:$A$181,"Base",'03_Calculation'!$B$2:$B$181,$A14,'03_Calculation'!$C$2:$C$181,B$5)/1000000000000000</f>
+        <v/>
+      </c>
+      <c r="C14" s="11">
+        <f>SUMIFS('03_Calculation'!$Y$2:$Y$181,'03_Calculation'!$A$2:$A$181,"Base",'03_Calculation'!$B$2:$B$181,$A14,'03_Calculation'!$C$2:$C$181,C$5)/1000000000000000</f>
+        <v/>
+      </c>
+      <c r="D14" s="11">
+        <f>SUMIFS('03_Calculation'!$Y$2:$Y$181,'03_Calculation'!$A$2:$A$181,"Base",'03_Calculation'!$B$2:$B$181,$A14,'03_Calculation'!$C$2:$C$181,D$5)/1000000000000000</f>
+        <v/>
+      </c>
+      <c r="E14" s="11">
+        <f>SUMIFS('03_Calculation'!$Y$2:$Y$181,'03_Calculation'!$A$2:$A$181,"Base",'03_Calculation'!$B$2:$B$181,$A14,'03_Calculation'!$C$2:$C$181,E$5)/1000000000000000</f>
+        <v/>
+      </c>
+      <c r="F14" s="11">
+        <f>SUMIFS('03_Calculation'!$Y$2:$Y$181,'03_Calculation'!$A$2:$A$181,"Base",'03_Calculation'!$B$2:$B$181,$A14,'03_Calculation'!$C$2:$C$181,F$5)/1000000000000000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="15" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="B15" s="16">
+        <f>SUM(B6:B14)</f>
+        <v/>
+      </c>
+      <c r="C15" s="16">
+        <f>SUM(C6:C14)</f>
+        <v/>
+      </c>
+      <c r="D15" s="16">
+        <f>SUM(D6:D14)</f>
+        <v/>
+      </c>
+      <c r="E15" s="16">
+        <f>SUM(E6:E14)</f>
+        <v/>
+      </c>
+      <c r="F15" s="16">
+        <f>SUM(F6:F14)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="13" t="n"/>
+      <c r="B16" s="3" t="n"/>
+      <c r="C16" s="3" t="n"/>
+      <c r="D16" s="3" t="n"/>
+      <c r="E16" s="3" t="n"/>
+      <c r="F16" s="3" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>Base Provider Time Series - Generated Output Tokens/Year (Q)</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="n"/>
+      <c r="C17" s="3" t="n"/>
+      <c r="D17" s="3" t="n"/>
+      <c r="E17" s="3" t="n"/>
+      <c r="F17" s="3" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="14" t="inlineStr">
+        <is>
+          <t>Provider</t>
+        </is>
+      </c>
+      <c r="B18" s="14" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C18" s="14" t="n">
+        <v>2027</v>
+      </c>
+      <c r="D18" s="14" t="n">
+        <v>2028</v>
+      </c>
+      <c r="E18" s="14" t="n">
+        <v>2029</v>
+      </c>
+      <c r="F18" s="14" t="n">
+        <v>2030</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>Microsoft</t>
+        </is>
+      </c>
+      <c r="B19" s="11">
+        <f>SUMIFS('03_Calculation'!$Z$2:$Z$181,'03_Calculation'!$A$2:$A$181,"Base",'03_Calculation'!$B$2:$B$181,$A19,'03_Calculation'!$C$2:$C$181,B$18)/1000000000000000</f>
+        <v/>
+      </c>
+      <c r="C19" s="11">
+        <f>SUMIFS('03_Calculation'!$Z$2:$Z$181,'03_Calculation'!$A$2:$A$181,"Base",'03_Calculation'!$B$2:$B$181,$A19,'03_Calculation'!$C$2:$C$181,C$18)/1000000000000000</f>
+        <v/>
+      </c>
+      <c r="D19" s="11">
+        <f>SUMIFS('03_Calculation'!$Z$2:$Z$181,'03_Calculation'!$A$2:$A$181,"Base",'03_Calculation'!$B$2:$B$181,$A19,'03_Calculation'!$C$2:$C$181,D$18)/1000000000000000</f>
+        <v/>
+      </c>
+      <c r="E19" s="11">
+        <f>SUMIFS('03_Calculation'!$Z$2:$Z$181,'03_Calculation'!$A$2:$A$181,"Base",'03_Calculation'!$B$2:$B$181,$A19,'03_Calculation'!$C$2:$C$181,E$18)/1000000000000000</f>
+        <v/>
+      </c>
+      <c r="F19" s="11">
+        <f>SUMIFS('03_Calculation'!$Z$2:$Z$181,'03_Calculation'!$A$2:$A$181,"Base",'03_Calculation'!$B$2:$B$181,$A19,'03_Calculation'!$C$2:$C$181,F$18)/1000000000000000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>Google</t>
+        </is>
+      </c>
+      <c r="B20" s="11">
+        <f>SUMIFS('03_Calculation'!$Z$2:$Z$181,'03_Calculation'!$A$2:$A$181,"Base",'03_Calculation'!$B$2:$B$181,$A20,'03_Calculation'!$C$2:$C$181,B$18)/1000000000000000</f>
+        <v/>
+      </c>
+      <c r="C20" s="11">
+        <f>SUMIFS('03_Calculation'!$Z$2:$Z$181,'03_Calculation'!$A$2:$A$181,"Base",'03_Calculation'!$B$2:$B$181,$A20,'03_Calculation'!$C$2:$C$181,C$18)/1000000000000000</f>
+        <v/>
+      </c>
+      <c r="D20" s="11">
+        <f>SUMIFS('03_Calculation'!$Z$2:$Z$181,'03_Calculation'!$A$2:$A$181,"Base",'03_Calculation'!$B$2:$B$181,$A20,'03_Calculation'!$C$2:$C$181,D$18)/1000000000000000</f>
+        <v/>
+      </c>
+      <c r="E20" s="11">
+        <f>SUMIFS('03_Calculation'!$Z$2:$Z$181,'03_Calculation'!$A$2:$A$181,"Base",'03_Calculation'!$B$2:$B$181,$A20,'03_Calculation'!$C$2:$C$181,E$18)/1000000000000000</f>
+        <v/>
+      </c>
+      <c r="F20" s="11">
+        <f>SUMIFS('03_Calculation'!$Z$2:$Z$181,'03_Calculation'!$A$2:$A$181,"Base",'03_Calculation'!$B$2:$B$181,$A20,'03_Calculation'!$C$2:$C$181,F$18)/1000000000000000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>Meta</t>
+        </is>
+      </c>
+      <c r="B21" s="11">
+        <f>SUMIFS('03_Calculation'!$Z$2:$Z$181,'03_Calculation'!$A$2:$A$181,"Base",'03_Calculation'!$B$2:$B$181,$A21,'03_Calculation'!$C$2:$C$181,B$18)/1000000000000000</f>
+        <v/>
+      </c>
+      <c r="C21" s="11">
+        <f>SUMIFS('03_Calculation'!$Z$2:$Z$181,'03_Calculation'!$A$2:$A$181,"Base",'03_Calculation'!$B$2:$B$181,$A21,'03_Calculation'!$C$2:$C$181,C$18)/1000000000000000</f>
+        <v/>
+      </c>
+      <c r="D21" s="11">
+        <f>SUMIFS('03_Calculation'!$Z$2:$Z$181,'03_Calculation'!$A$2:$A$181,"Base",'03_Calculation'!$B$2:$B$181,$A21,'03_Calculation'!$C$2:$C$181,D$18)/1000000000000000</f>
+        <v/>
+      </c>
+      <c r="E21" s="11">
+        <f>SUMIFS('03_Calculation'!$Z$2:$Z$181,'03_Calculation'!$A$2:$A$181,"Base",'03_Calculation'!$B$2:$B$181,$A21,'03_Calculation'!$C$2:$C$181,E$18)/1000000000000000</f>
+        <v/>
+      </c>
+      <c r="F21" s="11">
+        <f>SUMIFS('03_Calculation'!$Z$2:$Z$181,'03_Calculation'!$A$2:$A$181,"Base",'03_Calculation'!$B$2:$B$181,$A21,'03_Calculation'!$C$2:$C$181,F$18)/1000000000000000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>xAI</t>
+        </is>
+      </c>
+      <c r="B22" s="11">
+        <f>SUMIFS('03_Calculation'!$Z$2:$Z$181,'03_Calculation'!$A$2:$A$181,"Base",'03_Calculation'!$B$2:$B$181,$A22,'03_Calculation'!$C$2:$C$181,B$18)/1000000000000000</f>
+        <v/>
+      </c>
+      <c r="C22" s="11">
+        <f>SUMIFS('03_Calculation'!$Z$2:$Z$181,'03_Calculation'!$A$2:$A$181,"Base",'03_Calculation'!$B$2:$B$181,$A22,'03_Calculation'!$C$2:$C$181,C$18)/1000000000000000</f>
+        <v/>
+      </c>
+      <c r="D22" s="11">
+        <f>SUMIFS('03_Calculation'!$Z$2:$Z$181,'03_Calculation'!$A$2:$A$181,"Base",'03_Calculation'!$B$2:$B$181,$A22,'03_Calculation'!$C$2:$C$181,D$18)/1000000000000000</f>
+        <v/>
+      </c>
+      <c r="E22" s="11">
+        <f>SUMIFS('03_Calculation'!$Z$2:$Z$181,'03_Calculation'!$A$2:$A$181,"Base",'03_Calculation'!$B$2:$B$181,$A22,'03_Calculation'!$C$2:$C$181,E$18)/1000000000000000</f>
+        <v/>
+      </c>
+      <c r="F22" s="11">
+        <f>SUMIFS('03_Calculation'!$Z$2:$Z$181,'03_Calculation'!$A$2:$A$181,"Base",'03_Calculation'!$B$2:$B$181,$A22,'03_Calculation'!$C$2:$C$181,F$18)/1000000000000000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>OpenAI</t>
+        </is>
+      </c>
+      <c r="B23" s="11">
+        <f>SUMIFS('03_Calculation'!$Z$2:$Z$181,'03_Calculation'!$A$2:$A$181,"Base",'03_Calculation'!$B$2:$B$181,$A23,'03_Calculation'!$C$2:$C$181,B$18)/1000000000000000</f>
+        <v/>
+      </c>
+      <c r="C23" s="11">
+        <f>SUMIFS('03_Calculation'!$Z$2:$Z$181,'03_Calculation'!$A$2:$A$181,"Base",'03_Calculation'!$B$2:$B$181,$A23,'03_Calculation'!$C$2:$C$181,C$18)/1000000000000000</f>
+        <v/>
+      </c>
+      <c r="D23" s="11">
+        <f>SUMIFS('03_Calculation'!$Z$2:$Z$181,'03_Calculation'!$A$2:$A$181,"Base",'03_Calculation'!$B$2:$B$181,$A23,'03_Calculation'!$C$2:$C$181,D$18)/1000000000000000</f>
+        <v/>
+      </c>
+      <c r="E23" s="11">
+        <f>SUMIFS('03_Calculation'!$Z$2:$Z$181,'03_Calculation'!$A$2:$A$181,"Base",'03_Calculation'!$B$2:$B$181,$A23,'03_Calculation'!$C$2:$C$181,E$18)/1000000000000000</f>
+        <v/>
+      </c>
+      <c r="F23" s="11">
+        <f>SUMIFS('03_Calculation'!$Z$2:$Z$181,'03_Calculation'!$A$2:$A$181,"Base",'03_Calculation'!$B$2:$B$181,$A23,'03_Calculation'!$C$2:$C$181,F$18)/1000000000000000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>Anthropic</t>
+        </is>
+      </c>
+      <c r="B24" s="11">
+        <f>SUMIFS('03_Calculation'!$Z$2:$Z$181,'03_Calculation'!$A$2:$A$181,"Base",'03_Calculation'!$B$2:$B$181,$A24,'03_Calculation'!$C$2:$C$181,B$18)/1000000000000000</f>
+        <v/>
+      </c>
+      <c r="C24" s="11">
+        <f>SUMIFS('03_Calculation'!$Z$2:$Z$181,'03_Calculation'!$A$2:$A$181,"Base",'03_Calculation'!$B$2:$B$181,$A24,'03_Calculation'!$C$2:$C$181,C$18)/1000000000000000</f>
+        <v/>
+      </c>
+      <c r="D24" s="11">
+        <f>SUMIFS('03_Calculation'!$Z$2:$Z$181,'03_Calculation'!$A$2:$A$181,"Base",'03_Calculation'!$B$2:$B$181,$A24,'03_Calculation'!$C$2:$C$181,D$18)/1000000000000000</f>
+        <v/>
+      </c>
+      <c r="E24" s="11">
+        <f>SUMIFS('03_Calculation'!$Z$2:$Z$181,'03_Calculation'!$A$2:$A$181,"Base",'03_Calculation'!$B$2:$B$181,$A24,'03_Calculation'!$C$2:$C$181,E$18)/1000000000000000</f>
+        <v/>
+      </c>
+      <c r="F24" s="11">
+        <f>SUMIFS('03_Calculation'!$Z$2:$Z$181,'03_Calculation'!$A$2:$A$181,"Base",'03_Calculation'!$B$2:$B$181,$A24,'03_Calculation'!$C$2:$C$181,F$18)/1000000000000000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>DeepSeek</t>
+        </is>
+      </c>
+      <c r="B25" s="11">
+        <f>SUMIFS('03_Calculation'!$Z$2:$Z$181,'03_Calculation'!$A$2:$A$181,"Base",'03_Calculation'!$B$2:$B$181,$A25,'03_Calculation'!$C$2:$C$181,B$18)/1000000000000000</f>
+        <v/>
+      </c>
+      <c r="C25" s="11">
+        <f>SUMIFS('03_Calculation'!$Z$2:$Z$181,'03_Calculation'!$A$2:$A$181,"Base",'03_Calculation'!$B$2:$B$181,$A25,'03_Calculation'!$C$2:$C$181,C$18)/1000000000000000</f>
+        <v/>
+      </c>
+      <c r="D25" s="11">
+        <f>SUMIFS('03_Calculation'!$Z$2:$Z$181,'03_Calculation'!$A$2:$A$181,"Base",'03_Calculation'!$B$2:$B$181,$A25,'03_Calculation'!$C$2:$C$181,D$18)/1000000000000000</f>
+        <v/>
+      </c>
+      <c r="E25" s="11">
+        <f>SUMIFS('03_Calculation'!$Z$2:$Z$181,'03_Calculation'!$A$2:$A$181,"Base",'03_Calculation'!$B$2:$B$181,$A25,'03_Calculation'!$C$2:$C$181,E$18)/1000000000000000</f>
+        <v/>
+      </c>
+      <c r="F25" s="11">
+        <f>SUMIFS('03_Calculation'!$Z$2:$Z$181,'03_Calculation'!$A$2:$A$181,"Base",'03_Calculation'!$B$2:$B$181,$A25,'03_Calculation'!$C$2:$C$181,F$18)/1000000000000000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>Alibaba</t>
+        </is>
+      </c>
+      <c r="B26" s="11">
+        <f>SUMIFS('03_Calculation'!$Z$2:$Z$181,'03_Calculation'!$A$2:$A$181,"Base",'03_Calculation'!$B$2:$B$181,$A26,'03_Calculation'!$C$2:$C$181,B$18)/1000000000000000</f>
+        <v/>
+      </c>
+      <c r="C26" s="11">
+        <f>SUMIFS('03_Calculation'!$Z$2:$Z$181,'03_Calculation'!$A$2:$A$181,"Base",'03_Calculation'!$B$2:$B$181,$A26,'03_Calculation'!$C$2:$C$181,C$18)/1000000000000000</f>
+        <v/>
+      </c>
+      <c r="D26" s="11">
+        <f>SUMIFS('03_Calculation'!$Z$2:$Z$181,'03_Calculation'!$A$2:$A$181,"Base",'03_Calculation'!$B$2:$B$181,$A26,'03_Calculation'!$C$2:$C$181,D$18)/1000000000000000</f>
+        <v/>
+      </c>
+      <c r="E26" s="11">
+        <f>SUMIFS('03_Calculation'!$Z$2:$Z$181,'03_Calculation'!$A$2:$A$181,"Base",'03_Calculation'!$B$2:$B$181,$A26,'03_Calculation'!$C$2:$C$181,E$18)/1000000000000000</f>
+        <v/>
+      </c>
+      <c r="F26" s="11">
+        <f>SUMIFS('03_Calculation'!$Z$2:$Z$181,'03_Calculation'!$A$2:$A$181,"Base",'03_Calculation'!$B$2:$B$181,$A26,'03_Calculation'!$C$2:$C$181,F$18)/1000000000000000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>Tencent</t>
+        </is>
+      </c>
+      <c r="B27" s="11">
+        <f>SUMIFS('03_Calculation'!$Z$2:$Z$181,'03_Calculation'!$A$2:$A$181,"Base",'03_Calculation'!$B$2:$B$181,$A27,'03_Calculation'!$C$2:$C$181,B$18)/1000000000000000</f>
+        <v/>
+      </c>
+      <c r="C27" s="11">
+        <f>SUMIFS('03_Calculation'!$Z$2:$Z$181,'03_Calculation'!$A$2:$A$181,"Base",'03_Calculation'!$B$2:$B$181,$A27,'03_Calculation'!$C$2:$C$181,C$18)/1000000000000000</f>
+        <v/>
+      </c>
+      <c r="D27" s="11">
+        <f>SUMIFS('03_Calculation'!$Z$2:$Z$181,'03_Calculation'!$A$2:$A$181,"Base",'03_Calculation'!$B$2:$B$181,$A27,'03_Calculation'!$C$2:$C$181,D$18)/1000000000000000</f>
+        <v/>
+      </c>
+      <c r="E27" s="11">
+        <f>SUMIFS('03_Calculation'!$Z$2:$Z$181,'03_Calculation'!$A$2:$A$181,"Base",'03_Calculation'!$B$2:$B$181,$A27,'03_Calculation'!$C$2:$C$181,E$18)/1000000000000000</f>
+        <v/>
+      </c>
+      <c r="F27" s="11">
+        <f>SUMIFS('03_Calculation'!$Z$2:$Z$181,'03_Calculation'!$A$2:$A$181,"Base",'03_Calculation'!$B$2:$B$181,$A27,'03_Calculation'!$C$2:$C$181,F$18)/1000000000000000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="15" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="B28" s="16">
+        <f>SUM(B19:B27)</f>
+        <v/>
+      </c>
+      <c r="C28" s="16">
+        <f>SUM(C19:C27)</f>
+        <v/>
+      </c>
+      <c r="D28" s="16">
+        <f>SUM(D19:D27)</f>
+        <v/>
+      </c>
+      <c r="E28" s="16">
+        <f>SUM(E19:E27)</f>
+        <v/>
+      </c>
+      <c r="F28" s="16">
+        <f>SUM(F19:F27)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="13" t="n"/>
+      <c r="B29" s="3" t="n"/>
+      <c r="C29" s="3" t="n"/>
+      <c r="D29" s="3" t="n"/>
+      <c r="E29" s="3" t="n"/>
+      <c r="F29" s="3" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="3" t="inlineStr">
+        <is>
+          <t>Scenario Total Time Series - Generated Output Tokens/Day (Q)</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n"/>
+      <c r="C30" s="3" t="n"/>
+      <c r="D30" s="3" t="n"/>
+      <c r="E30" s="3" t="n"/>
+      <c r="F30" s="3" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="14" t="inlineStr">
+        <is>
+          <t>Scenario</t>
+        </is>
+      </c>
+      <c r="B31" s="14" t="n">
+        <v>2026</v>
+      </c>
+      <c r="C31" s="14" t="n">
+        <v>2027</v>
+      </c>
+      <c r="D31" s="14" t="n">
+        <v>2028</v>
+      </c>
+      <c r="E31" s="14" t="n">
+        <v>2029</v>
+      </c>
+      <c r="F31" s="14" t="n">
+        <v>2030</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="3" t="inlineStr">
         <is>
           <t>Bear</t>
         </is>
       </c>
-      <c r="C13" s="15" t="inlineStr">
+      <c r="B32" s="11">
+        <f>SUMIFS('03_Calculation'!$Y$2:$Y$181,'03_Calculation'!$A$2:$A$181,$A32,'03_Calculation'!$C$2:$C$181,B$31)/1000000000000000</f>
+        <v/>
+      </c>
+      <c r="C32" s="11">
+        <f>SUMIFS('03_Calculation'!$Y$2:$Y$181,'03_Calculation'!$A$2:$A$181,$A32,'03_Calculation'!$C$2:$C$181,C$31)/1000000000000000</f>
+        <v/>
+      </c>
+      <c r="D32" s="11">
+        <f>SUMIFS('03_Calculation'!$Y$2:$Y$181,'03_Calculation'!$A$2:$A$181,$A32,'03_Calculation'!$C$2:$C$181,D$31)/1000000000000000</f>
+        <v/>
+      </c>
+      <c r="E32" s="11">
+        <f>SUMIFS('03_Calculation'!$Y$2:$Y$181,'03_Calculation'!$A$2:$A$181,$A32,'03_Calculation'!$C$2:$C$181,E$31)/1000000000000000</f>
+        <v/>
+      </c>
+      <c r="F32" s="11">
+        <f>SUMIFS('03_Calculation'!$Y$2:$Y$181,'03_Calculation'!$A$2:$A$181,$A32,'03_Calculation'!$C$2:$C$181,F$31)/1000000000000000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="inlineStr">
         <is>
           <t>Base</t>
         </is>
       </c>
-      <c r="D13" s="15" t="inlineStr">
+      <c r="B33" s="11">
+        <f>SUMIFS('03_Calculation'!$Y$2:$Y$181,'03_Calculation'!$A$2:$A$181,$A33,'03_Calculation'!$C$2:$C$181,B$31)/1000000000000000</f>
+        <v/>
+      </c>
+      <c r="C33" s="11">
+        <f>SUMIFS('03_Calculation'!$Y$2:$Y$181,'03_Calculation'!$A$2:$A$181,$A33,'03_Calculation'!$C$2:$C$181,C$31)/1000000000000000</f>
+        <v/>
+      </c>
+      <c r="D33" s="11">
+        <f>SUMIFS('03_Calculation'!$Y$2:$Y$181,'03_Calculation'!$A$2:$A$181,$A33,'03_Calculation'!$C$2:$C$181,D$31)/1000000000000000</f>
+        <v/>
+      </c>
+      <c r="E33" s="11">
+        <f>SUMIFS('03_Calculation'!$Y$2:$Y$181,'03_Calculation'!$A$2:$A$181,$A33,'03_Calculation'!$C$2:$C$181,E$31)/1000000000000000</f>
+        <v/>
+      </c>
+      <c r="F33" s="11">
+        <f>SUMIFS('03_Calculation'!$Y$2:$Y$181,'03_Calculation'!$A$2:$A$181,$A33,'03_Calculation'!$C$2:$C$181,F$31)/1000000000000000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="3" t="inlineStr">
         <is>
           <t>Bull</t>
         </is>
       </c>
-      <c r="E13" s="15" t="inlineStr">
+      <c r="B34" s="11">
+        <f>SUMIFS('03_Calculation'!$Y$2:$Y$181,'03_Calculation'!$A$2:$A$181,$A34,'03_Calculation'!$C$2:$C$181,B$31)/1000000000000000</f>
+        <v/>
+      </c>
+      <c r="C34" s="11">
+        <f>SUMIFS('03_Calculation'!$Y$2:$Y$181,'03_Calculation'!$A$2:$A$181,$A34,'03_Calculation'!$C$2:$C$181,C$31)/1000000000000000</f>
+        <v/>
+      </c>
+      <c r="D34" s="11">
+        <f>SUMIFS('03_Calculation'!$Y$2:$Y$181,'03_Calculation'!$A$2:$A$181,$A34,'03_Calculation'!$C$2:$C$181,D$31)/1000000000000000</f>
+        <v/>
+      </c>
+      <c r="E34" s="11">
+        <f>SUMIFS('03_Calculation'!$Y$2:$Y$181,'03_Calculation'!$A$2:$A$181,$A34,'03_Calculation'!$C$2:$C$181,E$31)/1000000000000000</f>
+        <v/>
+      </c>
+      <c r="F34" s="11">
+        <f>SUMIFS('03_Calculation'!$Y$2:$Y$181,'03_Calculation'!$A$2:$A$181,$A34,'03_Calculation'!$C$2:$C$181,F$31)/1000000000000000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="3" t="inlineStr">
         <is>
           <t>Grid-Constrained / Efficiency-Upside</t>
         </is>
       </c>
-      <c r="F13" s="3" t="n"/>
-      <c r="G13" s="3" t="n"/>
-    </row>
-    <row r="14">
-      <c r="A14" s="3" t="n">
+      <c r="B35" s="11">
+        <f>SUMIFS('03_Calculation'!$Y$2:$Y$181,'03_Calculation'!$A$2:$A$181,$A35,'03_Calculation'!$C$2:$C$181,B$31)/1000000000000000</f>
+        <v/>
+      </c>
+      <c r="C35" s="11">
+        <f>SUMIFS('03_Calculation'!$Y$2:$Y$181,'03_Calculation'!$A$2:$A$181,$A35,'03_Calculation'!$C$2:$C$181,C$31)/1000000000000000</f>
+        <v/>
+      </c>
+      <c r="D35" s="11">
+        <f>SUMIFS('03_Calculation'!$Y$2:$Y$181,'03_Calculation'!$A$2:$A$181,$A35,'03_Calculation'!$C$2:$C$181,D$31)/1000000000000000</f>
+        <v/>
+      </c>
+      <c r="E35" s="11">
+        <f>SUMIFS('03_Calculation'!$Y$2:$Y$181,'03_Calculation'!$A$2:$A$181,$A35,'03_Calculation'!$C$2:$C$181,E$31)/1000000000000000</f>
+        <v/>
+      </c>
+      <c r="F35" s="11">
+        <f>SUMIFS('03_Calculation'!$Y$2:$Y$181,'03_Calculation'!$A$2:$A$181,$A35,'03_Calculation'!$C$2:$C$181,F$31)/1000000000000000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="13" t="n"/>
+      <c r="B36" s="3" t="n"/>
+      <c r="C36" s="3" t="n"/>
+      <c r="D36" s="3" t="n"/>
+      <c r="E36" s="3" t="n"/>
+      <c r="F36" s="3" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="3" t="inlineStr">
+        <is>
+          <t>Scenario Total Time Series - Generated Output Tokens/Year (Q)</t>
+        </is>
+      </c>
+      <c r="B37" s="3" t="n"/>
+      <c r="C37" s="3" t="n"/>
+      <c r="D37" s="3" t="n"/>
+      <c r="E37" s="3" t="n"/>
+      <c r="F37" s="3" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="14" t="inlineStr">
+        <is>
+          <t>Scenario</t>
+        </is>
+      </c>
+      <c r="B38" s="14" t="n">
         <v>2026</v>
       </c>
-      <c r="B14" s="11">
-        <f>SUMIFS('03_Calculation'!$Y:$Y,'03_Calculation'!$A:$A,B$12,'03_Calculation'!$C:$C,$A14)/1000000000000000</f>
-        <v/>
-      </c>
-      <c r="C14" s="11">
-        <f>SUMIFS('03_Calculation'!$Y:$Y,'03_Calculation'!$A:$A,C$12,'03_Calculation'!$C:$C,$A14)/1000000000000000</f>
-        <v/>
-      </c>
-      <c r="D14" s="11">
-        <f>SUMIFS('03_Calculation'!$Y:$Y,'03_Calculation'!$A:$A,D$12,'03_Calculation'!$C:$C,$A14)/1000000000000000</f>
-        <v/>
-      </c>
-      <c r="E14" s="11">
-        <f>SUMIFS('03_Calculation'!$Y:$Y,'03_Calculation'!$A:$A,E$12,'03_Calculation'!$C:$C,$A14)/1000000000000000</f>
-        <v/>
-      </c>
-      <c r="F14" s="9" t="n"/>
-      <c r="G14" s="9" t="n"/>
-    </row>
-    <row r="15">
-      <c r="A15" s="3" t="n">
+      <c r="C38" s="14" t="n">
         <v>2027</v>
       </c>
-      <c r="B15" s="11">
-        <f>SUMIFS('03_Calculation'!$Y:$Y,'03_Calculation'!$A:$A,B$12,'03_Calculation'!$C:$C,$A15)/1000000000000000</f>
-        <v/>
-      </c>
-      <c r="C15" s="11">
-        <f>SUMIFS('03_Calculation'!$Y:$Y,'03_Calculation'!$A:$A,C$12,'03_Calculation'!$C:$C,$A15)/1000000000000000</f>
-        <v/>
-      </c>
-      <c r="D15" s="11">
-        <f>SUMIFS('03_Calculation'!$Y:$Y,'03_Calculation'!$A:$A,D$12,'03_Calculation'!$C:$C,$A15)/1000000000000000</f>
-        <v/>
-      </c>
-      <c r="E15" s="11">
-        <f>SUMIFS('03_Calculation'!$Y:$Y,'03_Calculation'!$A:$A,E$12,'03_Calculation'!$C:$C,$A15)/1000000000000000</f>
-        <v/>
-      </c>
-      <c r="F15" s="9" t="n"/>
-      <c r="G15" s="9" t="n"/>
-    </row>
-    <row r="16">
-      <c r="A16" s="3" t="n">
+      <c r="D38" s="14" t="n">
         <v>2028</v>
       </c>
-      <c r="B16" s="11">
-        <f>SUMIFS('03_Calculation'!$Y:$Y,'03_Calculation'!$A:$A,B$12,'03_Calculation'!$C:$C,$A16)/1000000000000000</f>
-        <v/>
-      </c>
-      <c r="C16" s="11">
-        <f>SUMIFS('03_Calculation'!$Y:$Y,'03_Calculation'!$A:$A,C$12,'03_Calculation'!$C:$C,$A16)/1000000000000000</f>
-        <v/>
-      </c>
-      <c r="D16" s="11">
-        <f>SUMIFS('03_Calculation'!$Y:$Y,'03_Calculation'!$A:$A,D$12,'03_Calculation'!$C:$C,$A16)/1000000000000000</f>
-        <v/>
-      </c>
-      <c r="E16" s="11">
-        <f>SUMIFS('03_Calculation'!$Y:$Y,'03_Calculation'!$A:$A,E$12,'03_Calculation'!$C:$C,$A16)/1000000000000000</f>
-        <v/>
-      </c>
-      <c r="F16" s="9" t="n"/>
-      <c r="G16" s="9" t="n"/>
-    </row>
-    <row r="17">
-      <c r="A17" s="3" t="n">
+      <c r="E38" s="14" t="n">
         <v>2029</v>
       </c>
-      <c r="B17" s="11">
-        <f>SUMIFS('03_Calculation'!$Y:$Y,'03_Calculation'!$A:$A,B$12,'03_Calculation'!$C:$C,$A17)/1000000000000000</f>
-        <v/>
-      </c>
-      <c r="C17" s="11">
-        <f>SUMIFS('03_Calculation'!$Y:$Y,'03_Calculation'!$A:$A,C$12,'03_Calculation'!$C:$C,$A17)/1000000000000000</f>
-        <v/>
-      </c>
-      <c r="D17" s="11">
-        <f>SUMIFS('03_Calculation'!$Y:$Y,'03_Calculation'!$A:$A,D$12,'03_Calculation'!$C:$C,$A17)/1000000000000000</f>
-        <v/>
-      </c>
-      <c r="E17" s="11">
-        <f>SUMIFS('03_Calculation'!$Y:$Y,'03_Calculation'!$A:$A,E$12,'03_Calculation'!$C:$C,$A17)/1000000000000000</f>
-        <v/>
-      </c>
-      <c r="F17" s="9" t="n"/>
-      <c r="G17" s="9" t="n"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="3" t="n">
+      <c r="F38" s="14" t="n">
         <v>2030</v>
       </c>
-      <c r="B18" s="11">
-        <f>SUMIFS('03_Calculation'!$Y:$Y,'03_Calculation'!$A:$A,B$12,'03_Calculation'!$C:$C,$A18)/1000000000000000</f>
-        <v/>
-      </c>
-      <c r="C18" s="11">
-        <f>SUMIFS('03_Calculation'!$Y:$Y,'03_Calculation'!$A:$A,C$12,'03_Calculation'!$C:$C,$A18)/1000000000000000</f>
-        <v/>
-      </c>
-      <c r="D18" s="11">
-        <f>SUMIFS('03_Calculation'!$Y:$Y,'03_Calculation'!$A:$A,D$12,'03_Calculation'!$C:$C,$A18)/1000000000000000</f>
-        <v/>
-      </c>
-      <c r="E18" s="11">
-        <f>SUMIFS('03_Calculation'!$Y:$Y,'03_Calculation'!$A:$A,E$12,'03_Calculation'!$C:$C,$A18)/1000000000000000</f>
-        <v/>
-      </c>
-      <c r="F18" s="9" t="n"/>
-      <c r="G18" s="9" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="3" t="inlineStr">
+        <is>
+          <t>Bear</t>
+        </is>
+      </c>
+      <c r="B39" s="11">
+        <f>SUMIFS('03_Calculation'!$Z$2:$Z$181,'03_Calculation'!$A$2:$A$181,$A39,'03_Calculation'!$C$2:$C$181,B$38)/1000000000000000</f>
+        <v/>
+      </c>
+      <c r="C39" s="11">
+        <f>SUMIFS('03_Calculation'!$Z$2:$Z$181,'03_Calculation'!$A$2:$A$181,$A39,'03_Calculation'!$C$2:$C$181,C$38)/1000000000000000</f>
+        <v/>
+      </c>
+      <c r="D39" s="11">
+        <f>SUMIFS('03_Calculation'!$Z$2:$Z$181,'03_Calculation'!$A$2:$A$181,$A39,'03_Calculation'!$C$2:$C$181,D$38)/1000000000000000</f>
+        <v/>
+      </c>
+      <c r="E39" s="11">
+        <f>SUMIFS('03_Calculation'!$Z$2:$Z$181,'03_Calculation'!$A$2:$A$181,$A39,'03_Calculation'!$C$2:$C$181,E$38)/1000000000000000</f>
+        <v/>
+      </c>
+      <c r="F39" s="11">
+        <f>SUMIFS('03_Calculation'!$Z$2:$Z$181,'03_Calculation'!$A$2:$A$181,$A39,'03_Calculation'!$C$2:$C$181,F$38)/1000000000000000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="3" t="inlineStr">
+        <is>
+          <t>Base</t>
+        </is>
+      </c>
+      <c r="B40" s="11">
+        <f>SUMIFS('03_Calculation'!$Z$2:$Z$181,'03_Calculation'!$A$2:$A$181,$A40,'03_Calculation'!$C$2:$C$181,B$38)/1000000000000000</f>
+        <v/>
+      </c>
+      <c r="C40" s="11">
+        <f>SUMIFS('03_Calculation'!$Z$2:$Z$181,'03_Calculation'!$A$2:$A$181,$A40,'03_Calculation'!$C$2:$C$181,C$38)/1000000000000000</f>
+        <v/>
+      </c>
+      <c r="D40" s="11">
+        <f>SUMIFS('03_Calculation'!$Z$2:$Z$181,'03_Calculation'!$A$2:$A$181,$A40,'03_Calculation'!$C$2:$C$181,D$38)/1000000000000000</f>
+        <v/>
+      </c>
+      <c r="E40" s="11">
+        <f>SUMIFS('03_Calculation'!$Z$2:$Z$181,'03_Calculation'!$A$2:$A$181,$A40,'03_Calculation'!$C$2:$C$181,E$38)/1000000000000000</f>
+        <v/>
+      </c>
+      <c r="F40" s="11">
+        <f>SUMIFS('03_Calculation'!$Z$2:$Z$181,'03_Calculation'!$A$2:$A$181,$A40,'03_Calculation'!$C$2:$C$181,F$38)/1000000000000000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="3" t="inlineStr">
+        <is>
+          <t>Bull</t>
+        </is>
+      </c>
+      <c r="B41" s="11">
+        <f>SUMIFS('03_Calculation'!$Z$2:$Z$181,'03_Calculation'!$A$2:$A$181,$A41,'03_Calculation'!$C$2:$C$181,B$38)/1000000000000000</f>
+        <v/>
+      </c>
+      <c r="C41" s="11">
+        <f>SUMIFS('03_Calculation'!$Z$2:$Z$181,'03_Calculation'!$A$2:$A$181,$A41,'03_Calculation'!$C$2:$C$181,C$38)/1000000000000000</f>
+        <v/>
+      </c>
+      <c r="D41" s="11">
+        <f>SUMIFS('03_Calculation'!$Z$2:$Z$181,'03_Calculation'!$A$2:$A$181,$A41,'03_Calculation'!$C$2:$C$181,D$38)/1000000000000000</f>
+        <v/>
+      </c>
+      <c r="E41" s="11">
+        <f>SUMIFS('03_Calculation'!$Z$2:$Z$181,'03_Calculation'!$A$2:$A$181,$A41,'03_Calculation'!$C$2:$C$181,E$38)/1000000000000000</f>
+        <v/>
+      </c>
+      <c r="F41" s="11">
+        <f>SUMIFS('03_Calculation'!$Z$2:$Z$181,'03_Calculation'!$A$2:$A$181,$A41,'03_Calculation'!$C$2:$C$181,F$38)/1000000000000000</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="3" t="inlineStr">
+        <is>
+          <t>Grid-Constrained / Efficiency-Upside</t>
+        </is>
+      </c>
+      <c r="B42" s="11">
+        <f>SUMIFS('03_Calculation'!$Z$2:$Z$181,'03_Calculation'!$A$2:$A$181,$A42,'03_Calculation'!$C$2:$C$181,B$38)/1000000000000000</f>
+        <v/>
+      </c>
+      <c r="C42" s="11">
+        <f>SUMIFS('03_Calculation'!$Z$2:$Z$181,'03_Calculation'!$A$2:$A$181,$A42,'03_Calculation'!$C$2:$C$181,C$38)/1000000000000000</f>
+        <v/>
+      </c>
+      <c r="D42" s="11">
+        <f>SUMIFS('03_Calculation'!$Z$2:$Z$181,'03_Calculation'!$A$2:$A$181,$A42,'03_Calculation'!$C$2:$C$181,D$38)/1000000000000000</f>
+        <v/>
+      </c>
+      <c r="E42" s="11">
+        <f>SUMIFS('03_Calculation'!$Z$2:$Z$181,'03_Calculation'!$A$2:$A$181,$A42,'03_Calculation'!$C$2:$C$181,E$38)/1000000000000000</f>
+        <v/>
+      </c>
+      <c r="F42" s="11">
+        <f>SUMIFS('03_Calculation'!$Z$2:$Z$181,'03_Calculation'!$A$2:$A$181,$A42,'03_Calculation'!$C$2:$C$181,F$38)/1000000000000000</f>
+        <v/>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:G1"/>
+  <mergeCells count="2">
+    <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A1:F1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
@@ -34778,7 +35637,7 @@
         <f>IF(SUMPRODUCT(--('03_Calculation'!$F$2:$F$181&gt;'03_Calculation'!$D$2:$D$181))=0,"PASS","FAIL")</f>
         <v/>
       </c>
-      <c r="C2" s="16">
+      <c r="C2" s="17">
         <f>B2</f>
         <v/>
       </c>
@@ -34793,7 +35652,7 @@
         <f>IF(SUMPRODUCT(--(ABS('03_Calculation'!$J$2:$J$181-('03_Calculation'!$L$2:$L$181+'03_Calculation'!$M$2:$M$181))&gt;0.001))=0,"PASS","FAIL")</f>
         <v/>
       </c>
-      <c r="C3" s="16">
+      <c r="C3" s="17">
         <f>B3</f>
         <v/>
       </c>
@@ -34808,7 +35667,7 @@
         <f>IF(SUMPRODUCT(--(ABS(1-('03_Calculation'!$N$2:$N$181+'03_Calculation'!$O$2:$O$181+'03_Calculation'!$P$2:$P$181+'03_Calculation'!$Q$2:$Q$181))&gt;0.002))=0,"PASS","FAIL")</f>
         <v/>
       </c>
-      <c r="C4" s="16">
+      <c r="C4" s="17">
         <f>B4</f>
         <v/>
       </c>
@@ -34823,7 +35682,7 @@
         <f>IF(AND(MIN('02_Inputs'!$K$2:$K$181)&gt;0,MAX('02_Inputs'!$K$2:$K$181)&lt;=1),"PASS","FAIL")</f>
         <v/>
       </c>
-      <c r="C5" s="16">
+      <c r="C5" s="17">
         <f>B5</f>
         <v/>
       </c>
@@ -34838,7 +35697,7 @@
         <f>IF(SUMPRODUCT(--(ABS('03_Calculation'!$X$2:$X$181-('03_Calculation'!$W$2:$W$181*'03_Calculation'!$V$2:$V$181))&gt;0.01))=0,"PASS","FAIL")</f>
         <v/>
       </c>
-      <c r="C6" s="16">
+      <c r="C6" s="17">
         <f>B6</f>
         <v/>
       </c>
@@ -34853,7 +35712,7 @@
         <f>IF(SUMPRODUCT(--('01_Benchmark_Input'!$J$2:$J$10&lt;&gt;'01_Benchmark_Input'!$F$2:$F$10))=0,"PASS","FAIL")</f>
         <v/>
       </c>
-      <c r="C7" s="16">
+      <c r="C7" s="17">
         <f>B7</f>
         <v/>
       </c>
@@ -34868,7 +35727,7 @@
         <f>"PASS - formula uses inference GW x fleet-weighted serving TPS/MW x seconds/day only"</f>
         <v/>
       </c>
-      <c r="C8" s="16">
+      <c r="C8" s="17">
         <f>B8</f>
         <v/>
       </c>
@@ -34913,73 +35772,73 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="13" t="inlineStr">
+      <c r="A3" s="18" t="inlineStr">
         <is>
           <t>Provider</t>
         </is>
       </c>
-      <c r="B3" s="13" t="inlineStr">
+      <c r="B3" s="18" t="inlineStr">
         <is>
           <t>Base 2030 Q/day</t>
         </is>
       </c>
-      <c r="C3" s="13" t="inlineStr">
+      <c r="C3" s="18" t="inlineStr">
         <is>
           <t>Bull 2030 Q/day</t>
         </is>
       </c>
-      <c r="D3" s="13" t="inlineStr">
+      <c r="D3" s="18" t="inlineStr">
         <is>
           <t>Bull vs Base</t>
         </is>
       </c>
-      <c r="E3" s="13" t="inlineStr">
+      <c r="E3" s="18" t="inlineStr">
         <is>
           <t>Bull Fit Factor</t>
         </is>
       </c>
-      <c r="F3" s="13" t="inlineStr">
+      <c r="F3" s="18" t="inlineStr">
         <is>
           <t>Bull Serving TPS/MW</t>
         </is>
       </c>
-      <c r="G3" s="13" t="inlineStr">
+      <c r="G3" s="18" t="inlineStr">
         <is>
           <t>Public Reference Ceiling Q/day</t>
         </is>
       </c>
-      <c r="H3" s="13" t="inlineStr">
+      <c r="H3" s="18" t="inlineStr">
         <is>
           <t>Required condition</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="17">
+      <c r="A4" s="19">
         <f>'03_Calculation'!B96</f>
         <v/>
       </c>
-      <c r="B4" s="18">
+      <c r="B4" s="20">
         <f>'03_Calculation'!Y51/1000000000000000</f>
         <v/>
       </c>
-      <c r="C4" s="18">
+      <c r="C4" s="20">
         <f>'03_Calculation'!Y96/1000000000000000</f>
         <v/>
       </c>
-      <c r="D4" s="19">
+      <c r="D4" s="21">
         <f>C4/B4-1</f>
         <v/>
       </c>
-      <c r="E4" s="19">
+      <c r="E4" s="21">
         <f>'03_Calculation'!V96</f>
         <v/>
       </c>
-      <c r="F4" s="17">
+      <c r="F4" s="19">
         <f>'03_Calculation'!X96</f>
         <v/>
       </c>
-      <c r="G4" s="18">
+      <c r="G4" s="20">
         <f>C4/E4</f>
         <v/>
       </c>
@@ -34990,31 +35849,31 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="17">
+      <c r="A5" s="19">
         <f>'03_Calculation'!B101</f>
         <v/>
       </c>
-      <c r="B5" s="18">
+      <c r="B5" s="20">
         <f>'03_Calculation'!Y56/1000000000000000</f>
         <v/>
       </c>
-      <c r="C5" s="18">
+      <c r="C5" s="20">
         <f>'03_Calculation'!Y101/1000000000000000</f>
         <v/>
       </c>
-      <c r="D5" s="19">
+      <c r="D5" s="21">
         <f>C5/B5-1</f>
         <v/>
       </c>
-      <c r="E5" s="19">
+      <c r="E5" s="21">
         <f>'03_Calculation'!V101</f>
         <v/>
       </c>
-      <c r="F5" s="17">
+      <c r="F5" s="19">
         <f>'03_Calculation'!X101</f>
         <v/>
       </c>
-      <c r="G5" s="18">
+      <c r="G5" s="20">
         <f>C5/E5</f>
         <v/>
       </c>
@@ -35025,31 +35884,31 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="17">
+      <c r="A6" s="19">
         <f>'03_Calculation'!B106</f>
         <v/>
       </c>
-      <c r="B6" s="18">
+      <c r="B6" s="20">
         <f>'03_Calculation'!Y61/1000000000000000</f>
         <v/>
       </c>
-      <c r="C6" s="18">
+      <c r="C6" s="20">
         <f>'03_Calculation'!Y106/1000000000000000</f>
         <v/>
       </c>
-      <c r="D6" s="19">
+      <c r="D6" s="21">
         <f>C6/B6-1</f>
         <v/>
       </c>
-      <c r="E6" s="19">
+      <c r="E6" s="21">
         <f>'03_Calculation'!V106</f>
         <v/>
       </c>
-      <c r="F6" s="17">
+      <c r="F6" s="19">
         <f>'03_Calculation'!X106</f>
         <v/>
       </c>
-      <c r="G6" s="18">
+      <c r="G6" s="20">
         <f>C6/E6</f>
         <v/>
       </c>
@@ -35060,31 +35919,31 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="17">
+      <c r="A7" s="19">
         <f>'03_Calculation'!B111</f>
         <v/>
       </c>
-      <c r="B7" s="18">
+      <c r="B7" s="20">
         <f>'03_Calculation'!Y66/1000000000000000</f>
         <v/>
       </c>
-      <c r="C7" s="18">
+      <c r="C7" s="20">
         <f>'03_Calculation'!Y111/1000000000000000</f>
         <v/>
       </c>
-      <c r="D7" s="19">
+      <c r="D7" s="21">
         <f>C7/B7-1</f>
         <v/>
       </c>
-      <c r="E7" s="19">
+      <c r="E7" s="21">
         <f>'03_Calculation'!V111</f>
         <v/>
       </c>
-      <c r="F7" s="17">
+      <c r="F7" s="19">
         <f>'03_Calculation'!X111</f>
         <v/>
       </c>
-      <c r="G7" s="18">
+      <c r="G7" s="20">
         <f>C7/E7</f>
         <v/>
       </c>
@@ -35095,31 +35954,31 @@
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="17">
+      <c r="A8" s="19">
         <f>'03_Calculation'!B116</f>
         <v/>
       </c>
-      <c r="B8" s="18">
+      <c r="B8" s="20">
         <f>'03_Calculation'!Y71/1000000000000000</f>
         <v/>
       </c>
-      <c r="C8" s="18">
+      <c r="C8" s="20">
         <f>'03_Calculation'!Y116/1000000000000000</f>
         <v/>
       </c>
-      <c r="D8" s="19">
+      <c r="D8" s="21">
         <f>C8/B8-1</f>
         <v/>
       </c>
-      <c r="E8" s="19">
+      <c r="E8" s="21">
         <f>'03_Calculation'!V116</f>
         <v/>
       </c>
-      <c r="F8" s="17">
+      <c r="F8" s="19">
         <f>'03_Calculation'!X116</f>
         <v/>
       </c>
-      <c r="G8" s="18">
+      <c r="G8" s="20">
         <f>C8/E8</f>
         <v/>
       </c>
@@ -35130,31 +35989,31 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="17">
+      <c r="A9" s="19">
         <f>'03_Calculation'!B121</f>
         <v/>
       </c>
-      <c r="B9" s="18">
+      <c r="B9" s="20">
         <f>'03_Calculation'!Y76/1000000000000000</f>
         <v/>
       </c>
-      <c r="C9" s="18">
+      <c r="C9" s="20">
         <f>'03_Calculation'!Y121/1000000000000000</f>
         <v/>
       </c>
-      <c r="D9" s="19">
+      <c r="D9" s="21">
         <f>C9/B9-1</f>
         <v/>
       </c>
-      <c r="E9" s="19">
+      <c r="E9" s="21">
         <f>'03_Calculation'!V121</f>
         <v/>
       </c>
-      <c r="F9" s="17">
+      <c r="F9" s="19">
         <f>'03_Calculation'!X121</f>
         <v/>
       </c>
-      <c r="G9" s="18">
+      <c r="G9" s="20">
         <f>C9/E9</f>
         <v/>
       </c>
@@ -35165,31 +36024,31 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="17">
+      <c r="A10" s="19">
         <f>'03_Calculation'!B126</f>
         <v/>
       </c>
-      <c r="B10" s="18">
+      <c r="B10" s="20">
         <f>'03_Calculation'!Y81/1000000000000000</f>
         <v/>
       </c>
-      <c r="C10" s="18">
+      <c r="C10" s="20">
         <f>'03_Calculation'!Y126/1000000000000000</f>
         <v/>
       </c>
-      <c r="D10" s="19">
+      <c r="D10" s="21">
         <f>C10/B10-1</f>
         <v/>
       </c>
-      <c r="E10" s="19">
+      <c r="E10" s="21">
         <f>'03_Calculation'!V126</f>
         <v/>
       </c>
-      <c r="F10" s="17">
+      <c r="F10" s="19">
         <f>'03_Calculation'!X126</f>
         <v/>
       </c>
-      <c r="G10" s="18">
+      <c r="G10" s="20">
         <f>C10/E10</f>
         <v/>
       </c>
@@ -35200,31 +36059,31 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="17">
+      <c r="A11" s="19">
         <f>'03_Calculation'!B131</f>
         <v/>
       </c>
-      <c r="B11" s="18">
+      <c r="B11" s="20">
         <f>'03_Calculation'!Y86/1000000000000000</f>
         <v/>
       </c>
-      <c r="C11" s="18">
+      <c r="C11" s="20">
         <f>'03_Calculation'!Y131/1000000000000000</f>
         <v/>
       </c>
-      <c r="D11" s="19">
+      <c r="D11" s="21">
         <f>C11/B11-1</f>
         <v/>
       </c>
-      <c r="E11" s="19">
+      <c r="E11" s="21">
         <f>'03_Calculation'!V131</f>
         <v/>
       </c>
-      <c r="F11" s="17">
+      <c r="F11" s="19">
         <f>'03_Calculation'!X131</f>
         <v/>
       </c>
-      <c r="G11" s="18">
+      <c r="G11" s="20">
         <f>C11/E11</f>
         <v/>
       </c>
@@ -35235,31 +36094,31 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="17">
+      <c r="A12" s="19">
         <f>'03_Calculation'!B136</f>
         <v/>
       </c>
-      <c r="B12" s="18">
+      <c r="B12" s="20">
         <f>'03_Calculation'!Y91/1000000000000000</f>
         <v/>
       </c>
-      <c r="C12" s="18">
+      <c r="C12" s="20">
         <f>'03_Calculation'!Y136/1000000000000000</f>
         <v/>
       </c>
-      <c r="D12" s="19">
+      <c r="D12" s="21">
         <f>C12/B12-1</f>
         <v/>
       </c>
-      <c r="E12" s="19">
+      <c r="E12" s="21">
         <f>'03_Calculation'!V136</f>
         <v/>
       </c>
-      <c r="F12" s="17">
+      <c r="F12" s="19">
         <f>'03_Calculation'!X136</f>
         <v/>
       </c>
-      <c r="G12" s="18">
+      <c r="G12" s="20">
         <f>C12/E12</f>
         <v/>
       </c>
@@ -35270,14 +36129,14 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="13" t="n"/>
-      <c r="B13" s="13" t="n"/>
-      <c r="C13" s="13" t="n"/>
-      <c r="D13" s="13" t="n"/>
-      <c r="E13" s="13" t="n"/>
-      <c r="F13" s="13" t="n"/>
-      <c r="G13" s="13" t="n"/>
-      <c r="H13" s="13" t="n"/>
+      <c r="A13" s="18" t="n"/>
+      <c r="B13" s="18" t="n"/>
+      <c r="C13" s="18" t="n"/>
+      <c r="D13" s="18" t="n"/>
+      <c r="E13" s="18" t="n"/>
+      <c r="F13" s="18" t="n"/>
+      <c r="G13" s="18" t="n"/>
+      <c r="H13" s="18" t="n"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -35285,17 +36144,17 @@
           <t>Total Q generated output tokens/day</t>
         </is>
       </c>
-      <c r="B14" s="20" t="inlineStr">
+      <c r="B14" s="22" t="inlineStr">
         <is>
           <t>Base</t>
         </is>
       </c>
-      <c r="C14" s="20" t="inlineStr">
+      <c r="C14" s="22" t="inlineStr">
         <is>
           <t>Bull</t>
         </is>
       </c>
-      <c r="D14" s="20" t="inlineStr">
+      <c r="D14" s="22" t="inlineStr">
         <is>
           <t>Public Reference Ceiling</t>
         </is>
@@ -35305,106 +36164,106 @@
       <c r="A15" t="n">
         <v>2026</v>
       </c>
-      <c r="B15" s="18">
+      <c r="B15" s="20">
         <f>SUMIFS('03_Calculation'!$Y:$Y,'03_Calculation'!$A:$A,"Base",'03_Calculation'!$C:$C,$A15)/1000000000000000</f>
         <v/>
       </c>
-      <c r="C15" s="18">
+      <c r="C15" s="20">
         <f>SUMIFS('03_Calculation'!$Y:$Y,'03_Calculation'!$A:$A,"Bull",'03_Calculation'!$C:$C,$A15)/1000000000000000</f>
         <v/>
       </c>
-      <c r="D15" s="18">
+      <c r="D15" s="20">
         <f>SUMPRODUCT(('03_Calculation'!$A$2:$A$181="Bull")*('03_Calculation'!$C$2:$C$181=$A15)*('03_Calculation'!$Y$2:$Y$181/'03_Calculation'!$V$2:$V$181))/1000000000000000</f>
         <v/>
       </c>
-      <c r="E15" s="17" t="n"/>
-      <c r="F15" s="17" t="n"/>
-      <c r="G15" s="17" t="n"/>
-      <c r="H15" s="17" t="n"/>
+      <c r="E15" s="19" t="n"/>
+      <c r="F15" s="19" t="n"/>
+      <c r="G15" s="19" t="n"/>
+      <c r="H15" s="19" t="n"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
         <v>2027</v>
       </c>
-      <c r="B16" s="18">
+      <c r="B16" s="20">
         <f>SUMIFS('03_Calculation'!$Y:$Y,'03_Calculation'!$A:$A,"Base",'03_Calculation'!$C:$C,$A16)/1000000000000000</f>
         <v/>
       </c>
-      <c r="C16" s="18">
+      <c r="C16" s="20">
         <f>SUMIFS('03_Calculation'!$Y:$Y,'03_Calculation'!$A:$A,"Bull",'03_Calculation'!$C:$C,$A16)/1000000000000000</f>
         <v/>
       </c>
-      <c r="D16" s="18">
+      <c r="D16" s="20">
         <f>SUMPRODUCT(('03_Calculation'!$A$2:$A$181="Bull")*('03_Calculation'!$C$2:$C$181=$A16)*('03_Calculation'!$Y$2:$Y$181/'03_Calculation'!$V$2:$V$181))/1000000000000000</f>
         <v/>
       </c>
-      <c r="E16" s="17" t="n"/>
-      <c r="F16" s="17" t="n"/>
-      <c r="G16" s="17" t="n"/>
-      <c r="H16" s="17" t="n"/>
+      <c r="E16" s="19" t="n"/>
+      <c r="F16" s="19" t="n"/>
+      <c r="G16" s="19" t="n"/>
+      <c r="H16" s="19" t="n"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
         <v>2028</v>
       </c>
-      <c r="B17" s="18">
+      <c r="B17" s="20">
         <f>SUMIFS('03_Calculation'!$Y:$Y,'03_Calculation'!$A:$A,"Base",'03_Calculation'!$C:$C,$A17)/1000000000000000</f>
         <v/>
       </c>
-      <c r="C17" s="18">
+      <c r="C17" s="20">
         <f>SUMIFS('03_Calculation'!$Y:$Y,'03_Calculation'!$A:$A,"Bull",'03_Calculation'!$C:$C,$A17)/1000000000000000</f>
         <v/>
       </c>
-      <c r="D17" s="18">
+      <c r="D17" s="20">
         <f>SUMPRODUCT(('03_Calculation'!$A$2:$A$181="Bull")*('03_Calculation'!$C$2:$C$181=$A17)*('03_Calculation'!$Y$2:$Y$181/'03_Calculation'!$V$2:$V$181))/1000000000000000</f>
         <v/>
       </c>
-      <c r="E17" s="17" t="n"/>
-      <c r="F17" s="17" t="n"/>
-      <c r="G17" s="17" t="n"/>
-      <c r="H17" s="17" t="n"/>
+      <c r="E17" s="19" t="n"/>
+      <c r="F17" s="19" t="n"/>
+      <c r="G17" s="19" t="n"/>
+      <c r="H17" s="19" t="n"/>
     </row>
     <row r="18">
       <c r="A18" t="n">
         <v>2029</v>
       </c>
-      <c r="B18" s="18">
+      <c r="B18" s="20">
         <f>SUMIFS('03_Calculation'!$Y:$Y,'03_Calculation'!$A:$A,"Base",'03_Calculation'!$C:$C,$A18)/1000000000000000</f>
         <v/>
       </c>
-      <c r="C18" s="18">
+      <c r="C18" s="20">
         <f>SUMIFS('03_Calculation'!$Y:$Y,'03_Calculation'!$A:$A,"Bull",'03_Calculation'!$C:$C,$A18)/1000000000000000</f>
         <v/>
       </c>
-      <c r="D18" s="18">
+      <c r="D18" s="20">
         <f>SUMPRODUCT(('03_Calculation'!$A$2:$A$181="Bull")*('03_Calculation'!$C$2:$C$181=$A18)*('03_Calculation'!$Y$2:$Y$181/'03_Calculation'!$V$2:$V$181))/1000000000000000</f>
         <v/>
       </c>
-      <c r="E18" s="17" t="n"/>
-      <c r="F18" s="17" t="n"/>
-      <c r="G18" s="17" t="n"/>
-      <c r="H18" s="17" t="n"/>
+      <c r="E18" s="19" t="n"/>
+      <c r="F18" s="19" t="n"/>
+      <c r="G18" s="19" t="n"/>
+      <c r="H18" s="19" t="n"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
         <v>2030</v>
       </c>
-      <c r="B19" s="18">
+      <c r="B19" s="20">
         <f>SUMIFS('03_Calculation'!$Y:$Y,'03_Calculation'!$A:$A,"Base",'03_Calculation'!$C:$C,$A19)/1000000000000000</f>
         <v/>
       </c>
-      <c r="C19" s="18">
+      <c r="C19" s="20">
         <f>SUMIFS('03_Calculation'!$Y:$Y,'03_Calculation'!$A:$A,"Bull",'03_Calculation'!$C:$C,$A19)/1000000000000000</f>
         <v/>
       </c>
-      <c r="D19" s="18">
+      <c r="D19" s="20">
         <f>SUMPRODUCT(('03_Calculation'!$A$2:$A$181="Bull")*('03_Calculation'!$C$2:$C$181=$A19)*('03_Calculation'!$Y$2:$Y$181/'03_Calculation'!$V$2:$V$181))/1000000000000000</f>
         <v/>
       </c>
-      <c r="E19" s="17" t="n"/>
-      <c r="F19" s="17" t="n"/>
-      <c r="G19" s="17" t="n"/>
-      <c r="H19" s="17" t="n"/>
+      <c r="E19" s="19" t="n"/>
+      <c r="F19" s="19" t="n"/>
+      <c r="G19" s="19" t="n"/>
+      <c r="H19" s="19" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
Refresh InferenceX database and main config filters
</commit_message>
<xml_diff>
--- a/llm_token_capacity_project/outputs/reports/llm_token_capacity_2026_2030.xlsx
+++ b/llm_token_capacity_project/outputs/reports/llm_token_capacity_2026_2030.xlsx
@@ -1477,7 +1477,7 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>InferenceX output_tok_s_mw p50; single_turn / ISL 1024 / OSL 1024. 50행 미만/미존재 조합은 B200 placeholder로 시작합니다.</t>
+          <t>InferenceX output_tok_s_mw p50; model별 main_framework/main_precision 고정 + single_turn / ISL 1024 / OSL 1024. 50행 미만/미존재 조합은 B200 placeholder로 시작합니다.</t>
         </is>
       </c>
     </row>
@@ -1618,7 +1618,7 @@
         </is>
       </c>
       <c r="D2" s="5" t="n">
-        <v>369352</v>
+        <v>369518</v>
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
@@ -1626,7 +1626,7 @@
         </is>
       </c>
       <c r="F2" s="5" t="n">
-        <v>724940</v>
+        <v>723458</v>
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
@@ -1634,7 +1634,7 @@
         </is>
       </c>
       <c r="H2" s="5" t="n">
-        <v>724940</v>
+        <v>723458</v>
       </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
@@ -1642,7 +1642,7 @@
         </is>
       </c>
       <c r="J2" s="5" t="n">
-        <v>724940</v>
+        <v>723458</v>
       </c>
       <c r="K2" s="6" t="n">
         <v>0.4</v>
@@ -1671,7 +1671,7 @@
         </is>
       </c>
       <c r="D3" s="5" t="n">
-        <v>369352</v>
+        <v>369518</v>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
@@ -1679,7 +1679,7 @@
         </is>
       </c>
       <c r="F3" s="5" t="n">
-        <v>724940</v>
+        <v>723458</v>
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
@@ -1687,7 +1687,7 @@
         </is>
       </c>
       <c r="H3" s="5" t="n">
-        <v>724940</v>
+        <v>723458</v>
       </c>
       <c r="I3" s="3" t="inlineStr">
         <is>
@@ -1695,7 +1695,7 @@
         </is>
       </c>
       <c r="J3" s="5" t="n">
-        <v>724940</v>
+        <v>723458</v>
       </c>
       <c r="K3" s="6" t="n">
         <v>0.4</v>
@@ -1724,7 +1724,7 @@
         </is>
       </c>
       <c r="D4" s="5" t="n">
-        <v>284640</v>
+        <v>202722</v>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
@@ -1732,7 +1732,7 @@
         </is>
       </c>
       <c r="F4" s="5" t="n">
-        <v>282860</v>
+        <v>200857</v>
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
@@ -1740,7 +1740,7 @@
         </is>
       </c>
       <c r="H4" s="5" t="n">
-        <v>282860</v>
+        <v>200857</v>
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
@@ -1748,7 +1748,7 @@
         </is>
       </c>
       <c r="J4" s="5" t="n">
-        <v>282860</v>
+        <v>200857</v>
       </c>
       <c r="K4" s="6" t="n">
         <v>0.75</v>
@@ -1777,7 +1777,7 @@
         </is>
       </c>
       <c r="D5" s="5" t="n">
-        <v>369352</v>
+        <v>369518</v>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
@@ -1785,7 +1785,7 @@
         </is>
       </c>
       <c r="F5" s="5" t="n">
-        <v>724940</v>
+        <v>723458</v>
       </c>
       <c r="G5" s="3" t="inlineStr">
         <is>
@@ -1793,7 +1793,7 @@
         </is>
       </c>
       <c r="H5" s="5" t="n">
-        <v>724940</v>
+        <v>723458</v>
       </c>
       <c r="I5" s="3" t="inlineStr">
         <is>
@@ -1801,7 +1801,7 @@
         </is>
       </c>
       <c r="J5" s="5" t="n">
-        <v>724940</v>
+        <v>723458</v>
       </c>
       <c r="K5" s="6" t="n">
         <v>0.35</v>
@@ -1830,7 +1830,7 @@
         </is>
       </c>
       <c r="D6" s="5" t="n">
-        <v>369352</v>
+        <v>369518</v>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
@@ -1838,7 +1838,7 @@
         </is>
       </c>
       <c r="F6" s="5" t="n">
-        <v>724940</v>
+        <v>723458</v>
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
@@ -1846,7 +1846,7 @@
         </is>
       </c>
       <c r="H6" s="5" t="n">
-        <v>724940</v>
+        <v>723458</v>
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
@@ -1854,7 +1854,7 @@
         </is>
       </c>
       <c r="J6" s="5" t="n">
-        <v>724940</v>
+        <v>723458</v>
       </c>
       <c r="K6" s="6" t="n">
         <v>0.3</v>
@@ -1883,7 +1883,7 @@
         </is>
       </c>
       <c r="D7" s="5" t="n">
-        <v>369352</v>
+        <v>369518</v>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
@@ -1891,7 +1891,7 @@
         </is>
       </c>
       <c r="F7" s="5" t="n">
-        <v>724940</v>
+        <v>723458</v>
       </c>
       <c r="G7" s="3" t="inlineStr">
         <is>
@@ -1899,7 +1899,7 @@
         </is>
       </c>
       <c r="H7" s="5" t="n">
-        <v>724940</v>
+        <v>723458</v>
       </c>
       <c r="I7" s="3" t="inlineStr">
         <is>
@@ -1907,7 +1907,7 @@
         </is>
       </c>
       <c r="J7" s="5" t="n">
-        <v>724940</v>
+        <v>723458</v>
       </c>
       <c r="K7" s="6" t="n">
         <v>0.3</v>
@@ -1936,7 +1936,7 @@
         </is>
       </c>
       <c r="D8" s="5" t="n">
-        <v>60574</v>
+        <v>62631</v>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
@@ -1944,7 +1944,7 @@
         </is>
       </c>
       <c r="F8" s="5" t="n">
-        <v>101245</v>
+        <v>65077</v>
       </c>
       <c r="G8" s="3" t="inlineStr">
         <is>
@@ -1952,15 +1952,15 @@
         </is>
       </c>
       <c r="H8" s="5" t="n">
-        <v>731323</v>
+        <v>65077</v>
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>Public reference selected</t>
+          <t>B200 placeholder - insufficient/missing matched rows; editable input</t>
         </is>
       </c>
       <c r="J8" s="5" t="n">
-        <v>101245</v>
+        <v>65077</v>
       </c>
       <c r="K8" s="6" t="n">
         <v>0.65</v>
@@ -1989,31 +1989,31 @@
         </is>
       </c>
       <c r="D9" s="5" t="n">
-        <v>179145</v>
+        <v>89934</v>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
+          <t>Public reference selected</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="n">
+        <v>178342</v>
+      </c>
+      <c r="G9" s="3" t="inlineStr">
+        <is>
+          <t>Public reference selected</t>
+        </is>
+      </c>
+      <c r="H9" s="5" t="n">
+        <v>178342</v>
+      </c>
+      <c r="I9" s="3" t="inlineStr">
+        <is>
           <t>B200 placeholder - insufficient/missing matched rows; editable input</t>
         </is>
       </c>
-      <c r="F9" s="5" t="n">
-        <v>179145</v>
-      </c>
-      <c r="G9" s="3" t="inlineStr">
-        <is>
-          <t>Public reference selected</t>
-        </is>
-      </c>
-      <c r="H9" s="5" t="n">
-        <v>179145</v>
-      </c>
-      <c r="I9" s="3" t="inlineStr">
-        <is>
-          <t>B200 placeholder - insufficient/missing matched rows; editable input</t>
-        </is>
-      </c>
       <c r="J9" s="5" t="n">
-        <v>179145</v>
+        <v>178342</v>
       </c>
       <c r="K9" s="6" t="n">
         <v>0.7</v>
@@ -2042,7 +2042,7 @@
         </is>
       </c>
       <c r="D10" s="5" t="n">
-        <v>369352</v>
+        <v>369518</v>
       </c>
       <c r="E10" s="3" t="inlineStr">
         <is>
@@ -2050,7 +2050,7 @@
         </is>
       </c>
       <c r="F10" s="5" t="n">
-        <v>724940</v>
+        <v>723458</v>
       </c>
       <c r="G10" s="3" t="inlineStr">
         <is>
@@ -2058,7 +2058,7 @@
         </is>
       </c>
       <c r="H10" s="5" t="n">
-        <v>724940</v>
+        <v>723458</v>
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
@@ -2066,7 +2066,7 @@
         </is>
       </c>
       <c r="J10" s="5" t="n">
-        <v>724940</v>
+        <v>723458</v>
       </c>
       <c r="K10" s="6" t="n">
         <v>0.4</v>

</xml_diff>